<commit_message>
Fix Airbnb check-in (4 PM) and check-out (11 AM) times
- Day 1: beach before check-in, Airbnb check-in at 4 PM
- Day 9: check out by 11 AM, then airport
- All references updated from "accommodation" to "Airbnb"

Co-Authored-By: Claude (claude-opus-4-6[1m]) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/maui_itinerary.xlsx
+++ b/maui_itinerary.xlsx
@@ -853,7 +853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1046,164 +1046,164 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Thu, Apr 30</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>12:30 PM</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Check into accommodation</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>12:30 – 3:30 PM</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Beach time at Kamaole Beach Park (before check-in)</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Kihei</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Beach / Water</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr"/>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>Airbnb check-in not until 4 PM — hit the beach first! Drop bags at car</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Thu, Apr 30</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Check into Airbnb</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>2777 South Kihei Rd, Kihei</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Logistics</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="10" t="n">
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Airbnb check-in: 4:00 PM</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Thu, Apr 30</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>1:30 – 4:00 PM</t>
-        </is>
-      </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>Beach relaxation at Kamaole Beach Park</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>Kihei</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="inlineStr">
-        <is>
-          <t>Beach / Water</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="inlineStr"/>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>Calm water, easy access — gentle wade &amp; relax for Brittany</t>
-        </is>
-      </c>
-      <c r="I6" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>4:30 PM</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Unpack, freshen up, settle in</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>2777 S Kihei Rd</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Thu, Apr 30</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Dinner at Hula Grill Ka'anapali</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Ka'anapali</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>Hula Grill</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>Order cooked fish (avoid raw/sushi for pregnancy)</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Fri, May 1</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>8:30 – 10:00 AM</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>Gentle snorkel at Napili Bay (turtles, calm water)</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>Napili Bay</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
-        <is>
-          <t>Beach / Water</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="inlineStr"/>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>Snorkeling OK if Brittany comfortable — no scuba</t>
-        </is>
-      </c>
-      <c r="I8" s="10" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1220,12 +1220,12 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>10:00 – 11:30 AM</t>
+          <t>8:30 – 10:00 AM</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Beach relaxation at Napili Bay</t>
+          <t>Gentle snorkel at Napili Bay (turtles, calm water)</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -1241,51 +1241,51 @@
       <c r="G9" s="11" t="inlineStr"/>
       <c r="H9" s="11" t="inlineStr">
         <is>
+          <t>Snorkeling OK if Brittany comfortable — no scuba</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Fri, May 1</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>10:00 – 11:30 AM</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Beach relaxation at Napili Bay</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Napili Bay</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Beach / Water</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr"/>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
           <t>Float, enjoy the turtles. Shade &amp; hydration for Brittany</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Fri, May 1</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>12:00 PM</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Lunch — poke bowls from Fish Market Maui</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Lahaina area</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Food / Dining</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr"/>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Get cooked options for Brittany (no raw ahi)</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1302,170 +1302,166 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Lunch — poke bowls from Fish Market Maui</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Lahaina area</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Food / Dining</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr"/>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Get cooked options for Brittany (no raw ahi)</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Fri, May 1</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
           <t>12:45 PM</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>Shave ice at Ululani's Hawaiian Shave Ice</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Lahaina or Kihei</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>Ululani's</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>Get ice cream base — Roselani macadamia nut!</t>
         </is>
       </c>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="n">
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Fri, May 1</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>1:30 – 3:30 PM</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>Explore Lahaina town — banyan tree, Front St, galleries</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>Lahaina</t>
         </is>
       </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>Cultural / Sightseeing</t>
         </is>
       </c>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>Maui Strong Fund</t>
         </is>
       </c>
-      <c r="H12" s="13" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>Easy walking. Be respectful of rebuilding efforts</t>
         </is>
       </c>
-      <c r="I12" s="12" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Fri, May 1</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Sunset dinner at Mala Ocean Tavern</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Lahaina</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
         <is>
           <t>Mala Ocean Tavern</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>Alt: Fleetwood's on Front St if reopened</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>Sat, May 2</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>3:45 AM</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
-        <is>
-          <t>Depart for Haleakala summit (~1.5–2 hr drive)</t>
-        </is>
-      </c>
-      <c r="E14" s="16" t="inlineStr">
-        <is>
-          <t>2777 S Kihei Rd</t>
-        </is>
-      </c>
-      <c r="F14" s="15" t="inlineStr">
-        <is>
-          <t>Must-Book</t>
-        </is>
-      </c>
-      <c r="G14" s="17" t="inlineStr">
-        <is>
-          <t>Recreation.gov Reservations</t>
-        </is>
-      </c>
-      <c r="H14" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ MUST RESERVE. Sunrise ~5:50 AM. Warm layers!</t>
-        </is>
-      </c>
-      <c r="I14" s="15" t="inlineStr">
+      <c r="I14" s="7" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1482,322 +1478,326 @@
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
+          <t>3:45 AM</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Depart for Haleakala summit (~1.5–2 hr drive)</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>2777 S Kihei Rd</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>Must-Book</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>Recreation.gov Reservations</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>⚠️ MUST RESERVE. Sunrise ~5:50 AM. Warm layers!</t>
+        </is>
+      </c>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Sat, May 2</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
           <t>5:30 – 6:15 AM</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D16" s="16" t="inlineStr">
         <is>
           <t>Watch sunrise at Haleakala summit</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>Haleakala National Park</t>
         </is>
       </c>
-      <c r="F15" s="15" t="inlineStr">
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G15" s="16" t="inlineStr"/>
-      <c r="H15" s="16" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr"/>
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>Limit to ~30 min at summit — thin air &amp; pregnancy. Leave if dizzy</t>
         </is>
       </c>
-      <c r="I15" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="n">
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Sat, May 2</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>8:30 AM</t>
         </is>
       </c>
-      <c r="D16" s="19" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>Drive Upcountry. Visit Ali'i Kula Lavender Farm.</t>
         </is>
       </c>
-      <c r="E16" s="19" t="inlineStr">
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>Kula</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>Nature / Hiking</t>
         </is>
       </c>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="G17" s="20" t="inlineStr">
         <is>
           <t>Ali'i Kula Lavender</t>
         </is>
       </c>
-      <c r="H16" s="19" t="inlineStr">
+      <c r="H17" s="19" t="inlineStr">
         <is>
           <t>Gentle walking, beautiful scenery</t>
         </is>
       </c>
-      <c r="I16" s="18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n">
+      <c r="I17" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Sat, May 2</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>10:00 AM</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Brunch at Grandma's Coffee House or Kula Bistro</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Upcountry</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr"/>
-      <c r="H17" s="8" t="inlineStr"/>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="n">
+      <c r="G18" s="8" t="inlineStr"/>
+      <c r="H18" s="8" t="inlineStr"/>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Sat, May 2</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>11:30 AM</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>Surfing Goat Dairy or MauiWine at Ulupalakua</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>Ulupalakua</t>
         </is>
       </c>
-      <c r="F18" s="12" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>Cultural / Sightseeing</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>MauiWine</t>
         </is>
       </c>
-      <c r="H18" s="13" t="inlineStr">
+      <c r="H19" s="13" t="inlineStr">
         <is>
           <t>Non-alcoholic tastings for Brittany. Goat dairy is fun!</t>
         </is>
       </c>
-      <c r="I18" s="12" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="n">
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Sat, May 2</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>1:30 PM</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Stop at Leoda's Kitchen &amp; Pie Shop on drive back</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>820 Olowalu Village Rd, Lahaina</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr"/>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr"/>
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>Famous pies — banana cream, macnut, savory pot pies</t>
         </is>
       </c>
-      <c r="I19" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="n">
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Sat, May 2</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>3:00 – 5:00 PM</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Nap / rest at accommodation (early wake-up recovery!)</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Nap / rest at Airbnb (early wake-up recovery!)</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>2777 S Kihei Rd</t>
         </is>
       </c>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="F21" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr"/>
-      <c r="H20" s="11" t="inlineStr">
+      <c r="G21" s="11" t="inlineStr"/>
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>You earned this nap</t>
         </is>
       </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="n">
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Sat, May 2</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>Easy dinner — pick up food &amp; eat at accommodation</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Easy dinner — pick up food &amp; eat at Airbnb</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>2777 S Kihei Rd</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G21" s="8" t="inlineStr"/>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr"/>
+      <c r="H22" s="8" t="inlineStr">
         <is>
           <t>Rest up for Road to Hana tomorrow</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Sun, May 3</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>7:00 AM</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Depart for Road to Hana. Pack snacks &amp; water!</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>2777 S Kihei Rd</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Logistics</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>Download audio tour app BEFORE leaving (needs wifi). Bring crackers, fruit, water for nausea</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I22" s="7" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1841,623 +1841,623 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="n">
+      <c r="A24" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Sun, May 3</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>7:00 AM</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Depart for Road to Hana. Pack snacks &amp; water!</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>2777 S Kihei Rd</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr"/>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Start audio tour. Bring crackers, fruit, water for nausea</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Sun, May 3</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>8:00 AM</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
+      <c r="D25" s="19" t="inlineStr">
         <is>
           <t>Twin Falls (Mile 2) — easy short walk</t>
         </is>
       </c>
-      <c r="E24" s="19" t="inlineStr">
+      <c r="E25" s="19" t="inlineStr">
         <is>
           <t>Mile 2, Hana Hwy</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr">
+      <c r="F25" s="18" t="inlineStr">
         <is>
           <t>Nature / Hiking</t>
         </is>
       </c>
-      <c r="G24" s="19" t="inlineStr"/>
-      <c r="H24" s="19" t="inlineStr">
+      <c r="G25" s="19" t="inlineStr"/>
+      <c r="H25" s="19" t="inlineStr">
         <is>
           <t>Short &amp; gentle walk, fine for pregnancy</t>
         </is>
       </c>
-      <c r="I24" s="18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="n">
+      <c r="I25" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>Sun, May 3</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>8:45 AM</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>Banana bread &amp; fruit smoothie at Halfway to Hana</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>Haiku / Hana Hwy</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G25" s="8" t="inlineStr"/>
-      <c r="H25" s="8" t="inlineStr">
-        <is>
-          <t>Fresh fruit smoothies + shave ice stop!</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="18" t="n">
+      <c r="G26" s="8" t="inlineStr"/>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Fresh fruit smoothies + shave ice!</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
         <is>
           <t>Sun, May 3</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C27" s="18" t="inlineStr">
         <is>
           <t>9:30 AM</t>
         </is>
       </c>
-      <c r="D26" s="19" t="inlineStr">
+      <c r="D27" s="19" t="inlineStr">
         <is>
           <t>Garden of Eden Arboretum (Mile 10)</t>
         </is>
       </c>
-      <c r="E26" s="19" t="inlineStr">
+      <c r="E27" s="19" t="inlineStr">
         <is>
           <t>Mile 10, Hana Hwy</t>
         </is>
       </c>
-      <c r="F26" s="18" t="inlineStr">
+      <c r="F27" s="18" t="inlineStr">
         <is>
           <t>Nature / Hiking</t>
         </is>
       </c>
-      <c r="G26" s="20" t="inlineStr">
+      <c r="G27" s="20" t="inlineStr">
         <is>
           <t>Garden of Eden</t>
         </is>
       </c>
-      <c r="H26" s="19" t="inlineStr">
+      <c r="H27" s="19" t="inlineStr">
         <is>
           <t>Flat walking paths — pregnancy friendly</t>
         </is>
       </c>
-      <c r="I26" s="18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="n">
+      <c r="I27" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Sun, May 3</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>10:45 AM</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Ke'anae Peninsula (Mile 16.5) — scenic viewpoint</t>
         </is>
       </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="E28" s="13" t="inlineStr">
         <is>
           <t>Mile 16.5, Hana Hwy</t>
         </is>
       </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Cultural / Sightseeing</t>
         </is>
       </c>
-      <c r="G27" s="13" t="inlineStr"/>
-      <c r="H27" s="13" t="inlineStr">
+      <c r="G28" s="13" t="inlineStr"/>
+      <c r="H28" s="13" t="inlineStr">
         <is>
           <t>Quick stop, beautiful views, no hiking needed</t>
         </is>
       </c>
-      <c r="I27" s="12" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="18" t="n">
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B28" s="18" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>Sun, May 3</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>11:15 AM</t>
         </is>
       </c>
-      <c r="D28" s="19" t="inlineStr">
+      <c r="D29" s="19" t="inlineStr">
         <is>
           <t>Upper Waikani Falls / Three Bears Falls (Mile 19)</t>
         </is>
       </c>
-      <c r="E28" s="19" t="inlineStr">
+      <c r="E29" s="19" t="inlineStr">
         <is>
           <t>Mile 19, Hana Hwy</t>
         </is>
       </c>
-      <c r="F28" s="18" t="inlineStr">
+      <c r="F29" s="18" t="inlineStr">
         <is>
           <t>Nature / Hiking</t>
         </is>
       </c>
-      <c r="G28" s="19" t="inlineStr"/>
-      <c r="H28" s="19" t="inlineStr">
+      <c r="G29" s="19" t="inlineStr"/>
+      <c r="H29" s="19" t="inlineStr">
         <is>
           <t>Viewable from the road / short walk</t>
         </is>
       </c>
-      <c r="I28" s="18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="15" t="n">
+      <c r="I29" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Sun, May 3</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>12:30 PM</t>
         </is>
       </c>
-      <c r="D29" s="16" t="inlineStr">
-        <is>
-          <t>Wai'anapanapa State Park �� black sand beach, sea caves</t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="inlineStr">
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>Wai'anapanapa State Park — black sand beach, sea caves</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>Hana</t>
         </is>
       </c>
-      <c r="F29" s="15" t="inlineStr">
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G29" s="17" t="inlineStr">
+      <c r="G30" s="17" t="inlineStr">
         <is>
           <t>Wai'anapanapa Reservations</t>
         </is>
       </c>
-      <c r="H29" s="16" t="inlineStr">
+      <c r="H30" s="16" t="inlineStr">
         <is>
           <t>⚠️ MUST RESERVE park entry. Turnaround point</t>
         </is>
       </c>
-      <c r="I29" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="n">
+      <c r="I30" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Sun, May 3</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>1:30 PM</t>
         </is>
       </c>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>Lunch at Braddah Hutts BBQ food truck</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>Hana</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G30" s="8" t="inlineStr"/>
-      <c r="H30" s="8" t="inlineStr">
+      <c r="G31" s="8" t="inlineStr"/>
+      <c r="H31" s="8" t="inlineStr">
         <is>
           <t>Grab food before heading back</t>
         </is>
       </c>
-      <c r="I30" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Sun, May 3</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>2:15 PM</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>Drive back (reverse route — familiar road is easier)</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>Hana Hwy</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F32" s="4" t="inlineStr">
         <is>
           <t>Logistics</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr"/>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>Take it slow, stop at missed spots. Brittany can rest/nap</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="n">
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>Sun, May 3</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Arrive back in Kihei. Easy dinner at accommodation or Nuka</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Arrive back. Easy dinner at Airbnb or Nuka</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>Kihei / 2777 S Kihei Rd</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G32" s="8" t="inlineStr"/>
-      <c r="H32" s="8" t="inlineStr">
+      <c r="G33" s="8" t="inlineStr"/>
+      <c r="H33" s="8" t="inlineStr">
         <is>
           <t>Low-key after a long drive day</t>
         </is>
       </c>
-      <c r="I32" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="n">
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>Mon, May 4</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>9:00 AM</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
-        <is>
-          <t>Sleep in! Lazy morning at the accommodation</t>
-        </is>
-      </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Sleep in! Lazy morning at the Airbnb</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>2777 S Kihei Rd</t>
         </is>
       </c>
-      <c r="F33" s="10" t="inlineStr">
+      <c r="F34" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G33" s="11" t="inlineStr"/>
-      <c r="H33" s="11" t="inlineStr">
+      <c r="G34" s="11" t="inlineStr"/>
+      <c r="H34" s="11" t="inlineStr">
         <is>
           <t>You earned it after Hana. No alarm</t>
         </is>
       </c>
-      <c r="I33" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="n">
+      <c r="I34" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>Mon, May 4</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>9:30 AM</t>
         </is>
       </c>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>Acai bowls at Wow Wow Hawaiian Lemonade</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>Kihei</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G34" s="8" t="inlineStr"/>
-      <c r="H34" s="8" t="inlineStr">
+      <c r="G35" s="8" t="inlineStr"/>
+      <c r="H35" s="8" t="inlineStr">
         <is>
           <t>Fresh lemonades + acai bowls. Great healthy breakfast</t>
         </is>
       </c>
-      <c r="I34" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="n">
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Mon, May 4</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>10:30 AM – 1:00 PM</t>
         </is>
       </c>
-      <c r="D35" s="11" t="inlineStr">
+      <c r="D36" s="11" t="inlineStr">
         <is>
           <t>Beach relaxation at Kamaole Beach III</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Kihei</t>
         </is>
       </c>
-      <c r="F35" s="10" t="inlineStr">
+      <c r="F36" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G35" s="11" t="inlineStr"/>
-      <c r="H35" s="11" t="inlineStr">
-        <is>
-          <t>Walk from accommodation. Calm water, lifeguards, shade trees</t>
-        </is>
-      </c>
-      <c r="I35" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="7" t="n">
+      <c r="G36" s="11" t="inlineStr"/>
+      <c r="H36" s="11" t="inlineStr">
+        <is>
+          <t>Walk from Airbnb. Calm water, lifeguards, shade trees</t>
+        </is>
+      </c>
+      <c r="I36" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>Mon, May 4</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>1:00 PM</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>Shave ice at Surfing Monkey Shave Ice</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>1881 S Kihei Rd, Kihei</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G36" s="8" t="inlineStr"/>
-      <c r="H36" s="8" t="inlineStr">
+      <c r="G37" s="8" t="inlineStr"/>
+      <c r="H37" s="8" t="inlineStr">
         <is>
           <t>Kona coffee flavor + vegan coconut milk ice cream option</t>
         </is>
       </c>
-      <c r="I36" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="10" t="n">
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>Mon, May 4</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>2:00 – 4:00 PM</t>
         </is>
       </c>
-      <c r="D37" s="11" t="inlineStr">
+      <c r="D38" s="11" t="inlineStr">
         <is>
           <t>Prenatal spa treatment or continued beach time</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Wailea / Kihei</t>
         </is>
       </c>
-      <c r="F37" s="10" t="inlineStr">
+      <c r="F38" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G37" s="11" t="inlineStr"/>
-      <c r="H37" s="11" t="inlineStr">
+      <c r="G38" s="11" t="inlineStr"/>
+      <c r="H38" s="11" t="inlineStr">
         <is>
           <t>Prenatal massage at a Wailea spa — Brittany's choice!</t>
         </is>
       </c>
-      <c r="I37" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>Mon, May 4</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>4:15 PM</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Fresh fruit &amp; acai at Hawaiian Moons Natural Foods</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Kihei</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>Food / Dining</t>
-        </is>
-      </c>
-      <c r="G38" s="8" t="inlineStr"/>
-      <c r="H38" s="8" t="inlineStr">
-        <is>
-          <t>Tropical acai bowl + stock up on healthy snacks</t>
-        </is>
-      </c>
-      <c r="I38" s="7" t="inlineStr">
+      <c r="I38" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2474,125 +2474,121 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
+          <t>4:15 PM</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Fresh fruit &amp; acai at Hawaiian Moons Natural Foods</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Kihei</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Food / Dining</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr"/>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>Tropical acai bowl + stock up on healthy snacks</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Mon, May 4</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="D39" s="8" t="inlineStr">
+      <c r="D40" s="8" t="inlineStr">
         <is>
           <t>Dinner at Monkeypod Kitchen (happy hour, live music)</t>
         </is>
       </c>
-      <c r="E39" s="8" t="inlineStr">
+      <c r="E40" s="8" t="inlineStr">
         <is>
           <t>Wailea</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G39" s="9" t="inlineStr">
+      <c r="G40" s="9" t="inlineStr">
         <is>
           <t>Monkeypod Kitchen</t>
         </is>
       </c>
-      <c r="H39" s="8" t="inlineStr">
+      <c r="H40" s="8" t="inlineStr">
         <is>
           <t>Great mocktails for Brittany!</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="15" t="n">
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B40" s="15" t="inlineStr">
+      <c r="B41" s="15" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C40" s="15" t="inlineStr">
+      <c r="C41" s="15" t="inlineStr">
         <is>
           <t>6:00 AM</t>
         </is>
       </c>
-      <c r="D40" s="16" t="inlineStr">
+      <c r="D41" s="16" t="inlineStr">
         <is>
           <t>Molokini Crater snorkel boat tour (departs Ma'alaea)</t>
         </is>
       </c>
-      <c r="E40" s="16" t="inlineStr">
+      <c r="E41" s="16" t="inlineStr">
         <is>
           <t>Ma'alaea Harbor</t>
         </is>
       </c>
-      <c r="F40" s="15" t="inlineStr">
+      <c r="F41" s="15" t="inlineStr">
         <is>
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G40" s="17" t="inlineStr">
+      <c r="G41" s="17" t="inlineStr">
         <is>
           <t>Pacific Whale Foundation</t>
         </is>
       </c>
-      <c r="H40" s="16" t="inlineStr">
+      <c r="H41" s="16" t="inlineStr">
         <is>
           <t>⚠️ BOOK IN ADVANCE. Bring Dramamine (check w/ OB)</t>
         </is>
       </c>
-      <c r="I40" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Tue, May 5</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>11:30 AM</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>Lunch at Coconut's Fish Cafe</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>Kihei</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>Food / Dining</t>
-        </is>
-      </c>
-      <c r="G41" s="9" t="inlineStr">
-        <is>
-          <t>Coconut's Fish Cafe</t>
-        </is>
-      </c>
-      <c r="H41" s="8" t="inlineStr">
-        <is>
-          <t>Cooked fish tacos — pregnancy safe</t>
-        </is>
-      </c>
-      <c r="I41" s="7" t="inlineStr">
+      <c r="I41" s="15" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2609,412 +2605,416 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
+          <t>11:30 AM</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Lunch at Coconut's Fish Cafe</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Kihei</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>Food / Dining</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>Coconut's Fish Cafe</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>Cooked fish tacos — pregnancy safe</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Tue, May 5</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
           <t>12:15 PM</t>
         </is>
       </c>
-      <c r="D42" s="8" t="inlineStr">
+      <c r="D43" s="8" t="inlineStr">
         <is>
           <t>Shave ice at Peace Love Shave Ice</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
+      <c r="E43" s="8" t="inlineStr">
         <is>
           <t>Azeka Plaza, Kihei</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
+      <c r="F43" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G42" s="8" t="inlineStr"/>
-      <c r="H42" s="8" t="inlineStr">
+      <c r="G43" s="8" t="inlineStr"/>
+      <c r="H43" s="8" t="inlineStr">
         <is>
           <t>Organic syrups, Thai Iced Tea flavor, Roselani ice cream base</t>
         </is>
       </c>
-      <c r="I42" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="18" t="n">
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="B43" s="18" t="inlineStr">
+      <c r="B44" s="18" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C43" s="18" t="inlineStr">
+      <c r="C44" s="18" t="inlineStr">
         <is>
           <t>1:00 PM</t>
         </is>
       </c>
-      <c r="D43" s="19" t="inlineStr">
+      <c r="D44" s="19" t="inlineStr">
         <is>
           <t>Visit Ahihi-Kinau Marine Preserve — tide pools &amp; lava fields</t>
         </is>
       </c>
-      <c r="E43" s="19" t="inlineStr">
+      <c r="E44" s="19" t="inlineStr">
         <is>
           <t>Wailea / La Perouse Bay</t>
         </is>
       </c>
-      <c r="F43" s="18" t="inlineStr">
+      <c r="F44" s="18" t="inlineStr">
         <is>
           <t>Nature / Hiking</t>
         </is>
       </c>
-      <c r="G43" s="19" t="inlineStr"/>
-      <c r="H43" s="19" t="inlineStr">
+      <c r="G44" s="19" t="inlineStr"/>
+      <c r="H44" s="19" t="inlineStr">
         <is>
           <t>Beautiful natural reserve. Gentle exploring, tide pools</t>
         </is>
       </c>
-      <c r="I43" s="18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="10" t="n">
+      <c r="I44" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B44" s="10" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C44" s="10" t="inlineStr">
+      <c r="C45" s="10" t="inlineStr">
         <is>
           <t>2:30 – 4:30 PM</t>
         </is>
       </c>
-      <c r="D44" s="11" t="inlineStr">
+      <c r="D45" s="11" t="inlineStr">
         <is>
           <t>Beach relaxation at Big Beach (Makena State Park)</t>
         </is>
       </c>
-      <c r="E44" s="11" t="inlineStr">
+      <c r="E45" s="11" t="inlineStr">
         <is>
           <t>Makena</t>
         </is>
       </c>
-      <c r="F44" s="10" t="inlineStr">
+      <c r="F45" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G44" s="11" t="inlineStr"/>
-      <c r="H44" s="11" t="inlineStr">
+      <c r="G45" s="11" t="inlineStr"/>
+      <c r="H45" s="11" t="inlineStr">
         <is>
           <t>Watch the bodyboarders! Brittany should wade gently — big shore break</t>
         </is>
       </c>
-      <c r="I44" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="15" t="n">
+      <c r="I45" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B45" s="15" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C45" s="15" t="inlineStr">
+      <c r="C46" s="15" t="inlineStr">
         <is>
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
+      <c r="D46" s="16" t="inlineStr">
         <is>
           <t>Dinner at Mama's Fish House</t>
         </is>
       </c>
-      <c r="E45" s="16" t="inlineStr">
+      <c r="E46" s="16" t="inlineStr">
         <is>
           <t>Pa'ia</t>
         </is>
       </c>
-      <c r="F45" s="15" t="inlineStr">
+      <c r="F46" s="15" t="inlineStr">
         <is>
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G45" s="17" t="inlineStr">
+      <c r="G46" s="17" t="inlineStr">
         <is>
           <t>Mama's Fish House</t>
         </is>
       </c>
-      <c r="H45" s="16" t="inlineStr">
+      <c r="H46" s="16" t="inlineStr">
         <is>
           <t>⚠️ RESERVE WELL IN ADVANCE. Order cooked dishes for Brittany</t>
         </is>
       </c>
-      <c r="I45" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="18" t="n">
+      <c r="I46" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="B46" s="18" t="inlineStr">
+      <c r="B47" s="18" t="inlineStr">
         <is>
           <t>Wed, May 6</t>
         </is>
       </c>
-      <c r="C46" s="18" t="inlineStr">
+      <c r="C47" s="18" t="inlineStr">
         <is>
           <t>8:30 AM</t>
         </is>
       </c>
-      <c r="D46" s="19" t="inlineStr">
+      <c r="D47" s="19" t="inlineStr">
         <is>
           <t>'Iao Valley State Monument — 'Iao Needle viewpoint walk</t>
         </is>
       </c>
-      <c r="E46" s="19" t="inlineStr">
+      <c r="E47" s="19" t="inlineStr">
         <is>
           <t>'Iao Valley</t>
         </is>
       </c>
-      <c r="F46" s="18" t="inlineStr">
+      <c r="F47" s="18" t="inlineStr">
         <is>
           <t>Nature / Hiking</t>
         </is>
       </c>
-      <c r="G46" s="20" t="inlineStr">
+      <c r="G47" s="20" t="inlineStr">
         <is>
           <t>'Iao Valley Info</t>
         </is>
       </c>
-      <c r="H46" s="19" t="inlineStr">
+      <c r="H47" s="19" t="inlineStr">
         <is>
           <t>Short paved path. Perfect for pregnancy</t>
         </is>
       </c>
-      <c r="I46" s="18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="7" t="n">
+      <c r="I47" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B48" s="7" t="inlineStr">
         <is>
           <t>Wed, May 6</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>10:30 AM</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr">
+      <c r="D48" s="8" t="inlineStr">
         <is>
           <t>Lunch at Sam Sato's (dry mein and manju)</t>
         </is>
       </c>
-      <c r="E47" s="8" t="inlineStr">
+      <c r="E48" s="8" t="inlineStr">
         <is>
           <t>Wailuku</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G47" s="8" t="inlineStr"/>
-      <c r="H47" s="8" t="inlineStr">
+      <c r="G48" s="8" t="inlineStr"/>
+      <c r="H48" s="8" t="inlineStr">
         <is>
           <t>Famous local spot — the manju is a must!</t>
         </is>
       </c>
-      <c r="I47" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="10" t="n">
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B48" s="10" t="inlineStr">
+      <c r="B49" s="10" t="inlineStr">
         <is>
           <t>Wed, May 6</t>
         </is>
       </c>
-      <c r="C48" s="10" t="inlineStr">
+      <c r="C49" s="10" t="inlineStr">
         <is>
           <t>12:00 – 4:00 PM</t>
         </is>
       </c>
-      <c r="D48" s="11" t="inlineStr">
+      <c r="D49" s="11" t="inlineStr">
         <is>
           <t>Beach relaxation or Wailea Beach Path walk</t>
         </is>
       </c>
-      <c r="E48" s="11" t="inlineStr">
+      <c r="E49" s="11" t="inlineStr">
         <is>
           <t>Wailea / Kihei</t>
         </is>
       </c>
-      <c r="F48" s="10" t="inlineStr">
+      <c r="F49" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G48" s="11" t="inlineStr"/>
-      <c r="H48" s="11" t="inlineStr">
+      <c r="G49" s="11" t="inlineStr"/>
+      <c r="H49" s="11" t="inlineStr">
         <is>
           <t>Flat oceanfront path or lazy afternoon at the beach</t>
         </is>
       </c>
-      <c r="I48" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="15" t="n">
+      <c r="I49" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="B49" s="15" t="inlineStr">
+      <c r="B50" s="15" t="inlineStr">
         <is>
           <t>Wed, May 6</t>
         </is>
       </c>
-      <c r="C49" s="15" t="inlineStr">
+      <c r="C50" s="15" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="D49" s="16" t="inlineStr">
+      <c r="D50" s="16" t="inlineStr">
         <is>
           <t>Luau — Old Lahaina Luau or Feast at Lele</t>
         </is>
       </c>
-      <c r="E49" s="16" t="inlineStr">
+      <c r="E50" s="16" t="inlineStr">
         <is>
           <t>Lahaina</t>
         </is>
       </c>
-      <c r="F49" s="15" t="inlineStr">
+      <c r="F50" s="15" t="inlineStr">
         <is>
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G49" s="17" t="inlineStr">
+      <c r="G50" s="17" t="inlineStr">
         <is>
           <t>Old Lahaina Luau</t>
         </is>
       </c>
-      <c r="H49" s="16" t="inlineStr">
+      <c r="H50" s="16" t="inlineStr">
         <is>
           <t>⚠️ BOOK IN ADVANCE. Seated &amp; relaxed — perfect for pregnancy</t>
         </is>
       </c>
-      <c r="I49" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="10" t="n">
+      <c r="I50" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B50" s="10" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr">
         <is>
           <t>Thu, May 7</t>
         </is>
       </c>
-      <c r="C50" s="10" t="inlineStr">
+      <c r="C51" s="10" t="inlineStr">
         <is>
           <t>8:00 AM</t>
         </is>
       </c>
-      <c r="D50" s="11" t="inlineStr">
+      <c r="D51" s="11" t="inlineStr">
         <is>
           <t>Easy morning walk along Wailea Beach Path</t>
         </is>
       </c>
-      <c r="E50" s="11" t="inlineStr">
+      <c r="E51" s="11" t="inlineStr">
         <is>
           <t>Wailea</t>
         </is>
       </c>
-      <c r="F50" s="10" t="inlineStr">
+      <c r="F51" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G50" s="11" t="inlineStr"/>
-      <c r="H50" s="11" t="inlineStr">
+      <c r="G51" s="11" t="inlineStr"/>
+      <c r="H51" s="11" t="inlineStr">
         <is>
           <t>Flat oceanfront path, gorgeous views. Great gentle exercise</t>
         </is>
       </c>
-      <c r="I50" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>Thu, May 7</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>9:00 AM</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>Acai bowl at Brekkie Bowls food truck</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>Wailea</t>
-        </is>
-      </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Food / Dining</t>
-        </is>
-      </c>
-      <c r="G51" s="8" t="inlineStr"/>
-      <c r="H51" s="8" t="inlineStr">
-        <is>
-          <t>Superfood acai bowl — perfect pregnancy fuel!</t>
-        </is>
-      </c>
-      <c r="I51" s="7" t="inlineStr">
+      <c r="I51" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3031,17 +3031,17 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>10:30 AM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
         <is>
-          <t>Shave ice at Ululani's (Kihei location)</t>
+          <t>Acai bowl at Brekkie Bowls food truck</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
-          <t>61 S Kihei Rd, Kihei</t>
+          <t>Wailea</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
@@ -3049,14 +3049,10 @@
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G52" s="9" t="inlineStr">
-        <is>
-          <t>Ululani's</t>
-        </is>
-      </c>
+      <c r="G52" s="8" t="inlineStr"/>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>Round 2! Try a different flavor combo</t>
+          <t>Superfood acai bowl — perfect pregnancy fuel!</t>
         </is>
       </c>
       <c r="I52" s="7" t="inlineStr">
@@ -3076,244 +3072,248 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
+          <t>10:30 AM</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Shave ice at Ululani's (Kihei location)</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>61 S Kihei Rd, Kihei</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>Food / Dining</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>Ululani's</t>
+        </is>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>Round 2! Try a different flavor combo</t>
+        </is>
+      </c>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Thu, May 7</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
           <t>11:15 AM</t>
         </is>
       </c>
-      <c r="D53" s="8" t="inlineStr">
+      <c r="D54" s="8" t="inlineStr">
         <is>
           <t>Fresh fruit bowls at Maui Fruit Ninja</t>
         </is>
       </c>
-      <c r="E53" s="8" t="inlineStr">
+      <c r="E54" s="8" t="inlineStr">
         <is>
           <t>Lahaina</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
+      <c r="F54" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G53" s="9" t="inlineStr">
+      <c r="G54" s="9" t="inlineStr">
         <is>
           <t>Maui Fruit Ninja</t>
         </is>
       </c>
-      <c r="H53" s="8" t="inlineStr">
+      <c r="H54" s="8" t="inlineStr">
         <is>
           <t>Seasonal tropical fruit bowls &amp; dairy-free sorbets</t>
         </is>
       </c>
-      <c r="I53" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="10" t="n">
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B54" s="10" t="inlineStr">
+      <c r="B55" s="10" t="inlineStr">
         <is>
           <t>Thu, May 7</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
+      <c r="C55" s="10" t="inlineStr">
         <is>
           <t>12:30 – 3:00 PM</t>
         </is>
       </c>
-      <c r="D54" s="11" t="inlineStr">
+      <c r="D55" s="11" t="inlineStr">
         <is>
           <t>Beach time + revisits, shopping, souvenirs</t>
         </is>
       </c>
-      <c r="E54" s="11" t="inlineStr">
+      <c r="E55" s="11" t="inlineStr">
         <is>
           <t>Various / Kihei</t>
         </is>
       </c>
-      <c r="F54" s="10" t="inlineStr">
+      <c r="F55" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G54" s="11" t="inlineStr"/>
-      <c r="H54" s="11" t="inlineStr">
+      <c r="G55" s="11" t="inlineStr"/>
+      <c r="H55" s="11" t="inlineStr">
         <is>
           <t>Last full beach day! Soak it in</t>
         </is>
       </c>
-      <c r="I54" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="7" t="n">
+      <c r="I55" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B56" s="7" t="inlineStr">
         <is>
           <t>Thu, May 7</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C56" s="7" t="inlineStr">
         <is>
           <t>3:30 PM</t>
         </is>
       </c>
-      <c r="D55" s="8" t="inlineStr">
+      <c r="D56" s="8" t="inlineStr">
         <is>
           <t>Pie &amp; treats at Leoda's Kitchen and Pie Shop</t>
         </is>
       </c>
-      <c r="E55" s="8" t="inlineStr">
+      <c r="E56" s="8" t="inlineStr">
         <is>
           <t>820 Olowalu Village Rd, Lahaina</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
+      <c r="F56" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G55" s="8" t="inlineStr"/>
-      <c r="H55" s="8" t="inlineStr">
+      <c r="G56" s="8" t="inlineStr"/>
+      <c r="H56" s="8" t="inlineStr">
         <is>
           <t>Famous pies — banana cream, macnut, savory pot pies</t>
         </is>
       </c>
-      <c r="I55" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="15" t="n">
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B56" s="15" t="inlineStr">
+      <c r="B57" s="15" t="inlineStr">
         <is>
           <t>Thu, May 7</t>
         </is>
       </c>
-      <c r="C56" s="15" t="inlineStr">
+      <c r="C57" s="15" t="inlineStr">
         <is>
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
+      <c r="D57" s="16" t="inlineStr">
         <is>
           <t>Final sunset dinner at Merriman's Kapalua</t>
         </is>
       </c>
-      <c r="E56" s="16" t="inlineStr">
+      <c r="E57" s="16" t="inlineStr">
         <is>
           <t>Kapalua</t>
         </is>
       </c>
-      <c r="F56" s="15" t="inlineStr">
+      <c r="F57" s="15" t="inlineStr">
         <is>
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G56" s="17" t="inlineStr">
+      <c r="G57" s="17" t="inlineStr">
         <is>
           <t>Merriman's Kapalua</t>
         </is>
       </c>
-      <c r="H56" s="16" t="inlineStr">
+      <c r="H57" s="16" t="inlineStr">
         <is>
           <t>BOOKED — hoping for outdoor 5:30 seating (waitlisted). Keep checking!</t>
         </is>
       </c>
-      <c r="I56" s="15" t="inlineStr">
+      <c r="I57" s="15" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="10" t="n">
+    <row r="58">
+      <c r="A58" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B57" s="10" t="inlineStr">
+      <c r="B58" s="10" t="inlineStr">
         <is>
           <t>Fri, May 8</t>
         </is>
       </c>
-      <c r="C57" s="10" t="inlineStr">
+      <c r="C58" s="10" t="inlineStr">
         <is>
           <t>7:00 AM</t>
         </is>
       </c>
-      <c r="D57" s="11" t="inlineStr">
+      <c r="D58" s="11" t="inlineStr">
         <is>
           <t>Last morning beach walk at Kamaole Beach</t>
         </is>
       </c>
-      <c r="E57" s="11" t="inlineStr">
+      <c r="E58" s="11" t="inlineStr">
         <is>
           <t>Kihei</t>
         </is>
       </c>
-      <c r="F57" s="10" t="inlineStr">
+      <c r="F58" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G57" s="11" t="inlineStr"/>
-      <c r="H57" s="11" t="inlineStr">
+      <c r="G58" s="11" t="inlineStr"/>
+      <c r="H58" s="11" t="inlineStr">
         <is>
           <t>One last Maui sunrise moment</t>
         </is>
       </c>
-      <c r="I57" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>Fri, May 8</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>8:00 AM</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Pack up, check out. Return rental car at OGG.</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>2777 S Kihei Rd → OGG</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>Logistics</t>
-        </is>
-      </c>
-      <c r="G58" s="5" t="inlineStr"/>
-      <c r="H58" s="5" t="inlineStr">
-        <is>
-          <t>Airport is ~25 min from Kihei</t>
-        </is>
-      </c>
-      <c r="I58" s="4" t="inlineStr">
+      <c r="I58" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3330,34 +3330,75 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
+          <t>8:00 – 10:00 AM</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Pack up &amp; check out of Airbnb by 11 AM. Return rental car.</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>2777 S Kihei Rd → OGG</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr"/>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>Airbnb check-out: 11:00 AM. Airport is ~25 min from Kihei</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Fri, May 8</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
           <t>10:40 AM</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>Flight AS 978 OGG → SFO. Arrive 6:44 PM.</t>
         </is>
       </c>
-      <c r="E59" s="5" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>OGG Airport</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr">
         <is>
           <t>Logistics</t>
         </is>
       </c>
-      <c r="G59" s="5" t="inlineStr"/>
-      <c r="H59" s="5" t="inlineStr"/>
-      <c r="I59" s="4" t="inlineStr">
+      <c r="G60" s="5" t="inlineStr"/>
+      <c r="H60" s="5" t="inlineStr"/>
+      <c r="I60" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I59">
+  <conditionalFormatting sqref="I2:I60">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Y"</formula>
     </cfRule>
@@ -3368,25 +3409,25 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G45" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G49" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G52" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G56" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3399,7 +3440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B65"/>
+  <dimension ref="A1:B67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3465,7 +3506,7 @@
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>Accommodation</t>
+          <t>Airbnb</t>
         </is>
       </c>
       <c r="B6" s="24" t="inlineStr">
@@ -3477,35 +3518,43 @@
     <row r="7">
       <c r="A7" s="23" t="inlineStr">
         <is>
+          <t>Airbnb Check-in</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>4:00 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>Airbnb Check-out</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
           <t>Rental Car</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Pick up &amp; return at OGG Airport</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>🤰 PREGNANCY TRAVEL NOTES</t>
-        </is>
-      </c>
-      <c r="B9" s="22" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>• Avoid raw fish/sushi (ahi poke) — order cooked fish dishes</t>
-        </is>
-      </c>
-      <c r="B10" s="22" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="25" t="inlineStr">
-        <is>
-          <t>• Avoid scuba diving, zip-lining, parasailing, horseback riding</t>
         </is>
       </c>
       <c r="B11" s="22" t="n"/>
@@ -3513,7 +3562,7 @@
     <row r="12">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>• Snorkeling is generally OK — check with OB first</t>
+          <t>• Avoid raw fish/sushi (ahi poke) — order cooked fish dishes</t>
         </is>
       </c>
       <c r="B12" s="22" t="n"/>
@@ -3521,7 +3570,7 @@
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>• Haleakala summit: thin air, limit time to ~30 min, leave if dizzy</t>
+          <t>• Avoid scuba diving, zip-lining, parasailing, horseback riding</t>
         </is>
       </c>
       <c r="B13" s="22" t="n"/>
@@ -3529,7 +3578,7 @@
     <row r="14">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>• Stay hydrated — bring water everywhere, seek shade often</t>
+          <t>• Snorkeling is generally OK — check with OB first</t>
         </is>
       </c>
       <c r="B14" s="22" t="n"/>
@@ -3537,7 +3586,7 @@
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t>• Dramamine for boat/car sickness — check with OB for pregnancy-safe brand</t>
+          <t>• Haleakala summit: thin air, limit time to ~30 min, leave if dizzy</t>
         </is>
       </c>
       <c r="B15" s="22" t="n"/>
@@ -3545,7 +3594,7 @@
     <row r="16">
       <c r="A16" s="25" t="inlineStr">
         <is>
-          <t>• Road to Hana: take breaks often, go slow, carry snacks (helps nausea)</t>
+          <t>• Stay hydrated — bring water everywhere, seek shade often</t>
         </is>
       </c>
       <c r="B16" s="22" t="n"/>
@@ -3553,7 +3602,7 @@
     <row r="17">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>• Big Beach (Makena): watch shore break — wade gently, don't bodyboard</t>
+          <t>• Dramamine for boat/car sickness — check with OB for pregnancy-safe brand</t>
         </is>
       </c>
       <c r="B17" s="22" t="n"/>
@@ -3561,7 +3610,7 @@
     <row r="18">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>• Prenatal massage: request pregnancy-trained masseuse (2nd/3rd trimester only)</t>
+          <t>• Road to Hana: take breaks often, go slow, carry snacks (helps nausea)</t>
         </is>
       </c>
       <c r="B18" s="22" t="n"/>
@@ -3569,7 +3618,7 @@
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>• Book an aisle seat on the plane for bathroom access</t>
+          <t>• Big Beach (Makena): watch shore break — wade gently, don't bodyboard</t>
         </is>
       </c>
       <c r="B19" s="22" t="n"/>
@@ -3577,251 +3626,251 @@
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
+          <t>• Prenatal massage: request pregnancy-trained masseuse (2nd/3rd trimester only)</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>• Book an aisle seat on the plane for bathroom access</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
+        <is>
           <t>• Wear compression socks for flights to prevent swelling</t>
         </is>
       </c>
-      <c r="B20" s="22" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="B22" s="22" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
         <is>
           <t>⚠️ MUST-BOOK IN ADVANCE ITEMS</t>
         </is>
       </c>
-      <c r="B22" s="22" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="26" t="inlineStr">
-        <is>
-          <t>Haleakala Sunrise Reservation</t>
-        </is>
-      </c>
-      <c r="B23" s="27" t="inlineStr">
-        <is>
-          <t>https://www.recreation.gov/ticket/facility/253731</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="26" t="inlineStr">
-        <is>
-          <t>Wai'anapanapa State Park Entry</t>
-        </is>
-      </c>
-      <c r="B24" s="27" t="inlineStr">
-        <is>
-          <t>https://www.gowaianapanapa.com/</t>
-        </is>
-      </c>
+      <c r="B24" s="22" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="26" t="inlineStr">
         <is>
-          <t>Molokini Snorkel Tour</t>
+          <t>Haleakala Sunrise Reservation</t>
         </is>
       </c>
       <c r="B25" s="27" t="inlineStr">
         <is>
-          <t>https://www.pacificwhale.org/cruises/molokini-snorkel/</t>
+          <t>https://www.recreation.gov/ticket/facility/253731</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>Mama's Fish House Dinner</t>
+          <t>Wai'anapanapa State Park Entry</t>
         </is>
       </c>
       <c r="B26" s="27" t="inlineStr">
         <is>
-          <t>https://www.mamasfishhouse.com/</t>
+          <t>https://www.gowaianapanapa.com/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>Old Lahaina Luau</t>
+          <t>Molokini Snorkel Tour</t>
         </is>
       </c>
       <c r="B27" s="27" t="inlineStr">
         <is>
-          <t>https://www.oldlahainaluau.com/</t>
+          <t>https://www.pacificwhale.org/cruises/molokini-snorkel/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="26" t="inlineStr">
         <is>
+          <t>Mama's Fish House Dinner</t>
+        </is>
+      </c>
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>https://www.mamasfishhouse.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t>Old Lahaina Luau</t>
+        </is>
+      </c>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>https://www.oldlahainaluau.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="26" t="inlineStr">
+        <is>
           <t>Merriman's Kapalua (BOOKED — waitlist outdoor 5:30)</t>
         </is>
       </c>
-      <c r="B28" s="27" t="inlineStr">
+      <c r="B30" s="27" t="inlineStr">
         <is>
           <t>https://www.merrimanshawaii.com/kapalua/</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
         <is>
           <t>🍧 SHAVED ICE / ACAI / FRUIT SPOTS</t>
         </is>
       </c>
-      <c r="B30" s="22" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="28" t="inlineStr">
-        <is>
-          <t>Ululani's Hawaiian Shave Ice</t>
-        </is>
-      </c>
-      <c r="B31" s="25" t="inlineStr">
-        <is>
-          <t>Kihei (61 S Kihei Rd), Kahului, Wailuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="28" t="inlineStr">
-        <is>
-          <t>Peace Love Shave Ice</t>
-        </is>
-      </c>
-      <c r="B32" s="25" t="inlineStr">
-        <is>
-          <t>Azeka Plaza, Kihei — organic syrups, Thai Iced Tea flavor</t>
-        </is>
-      </c>
+      <c r="B32" s="22" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="28" t="inlineStr">
         <is>
-          <t>Surfing Monkey Shave Ice</t>
+          <t>Ululani's Hawaiian Shave Ice</t>
         </is>
       </c>
       <c r="B33" s="25" t="inlineStr">
         <is>
-          <t>Kihei — Kona coffee flavor, vegan coconut milk ice cream</t>
+          <t>Kihei (61 S Kihei Rd), Kahului, Wailuku</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="28" t="inlineStr">
         <is>
-          <t>Halfway to Hana</t>
+          <t>Peace Love Shave Ice</t>
         </is>
       </c>
       <c r="B34" s="25" t="inlineStr">
         <is>
-          <t>Haiku — shave ice + banana bread on Hana Hwy</t>
+          <t>Azeka Plaza, Kihei — organic syrups, Thai Iced Tea flavor</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="28" t="inlineStr">
         <is>
-          <t>Mo'Ono Hawaii (food truck)</t>
+          <t>Surfing Monkey Shave Ice</t>
         </is>
       </c>
       <c r="B35" s="25" t="inlineStr">
         <is>
-          <t>Kahului — acai bowls, fresh fruit toppings</t>
+          <t>Kihei — Kona coffee flavor, vegan coconut milk ice cream</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="28" t="inlineStr">
         <is>
-          <t>Brekkie Bowls (food truck)</t>
+          <t>Halfway to Hana</t>
         </is>
       </c>
       <c r="B36" s="25" t="inlineStr">
         <is>
-          <t>Wailea — superfood acai bowls</t>
+          <t>Haiku — shave ice + banana bread on Hana Hwy</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="28" t="inlineStr">
         <is>
-          <t>Hawaiian Moons Natural Foods</t>
+          <t>Mo'Ono Hawaii (food truck)</t>
         </is>
       </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>Kihei — tropical acai bowl + healthy groceries</t>
+          <t>Kahului — acai bowls, fresh fruit toppings</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="28" t="inlineStr">
         <is>
-          <t>Wow Wow Hawaiian Lemonade</t>
+          <t>Brekkie Bowls (food truck)</t>
         </is>
       </c>
       <c r="B38" s="25" t="inlineStr">
         <is>
-          <t>Kihei — acai bowls + fresh lemonades</t>
+          <t>Wailea — superfood acai bowls</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="28" t="inlineStr">
         <is>
-          <t>Maui Fruit Ninja</t>
+          <t>Hawaiian Moons Natural Foods</t>
         </is>
       </c>
       <c r="B39" s="25" t="inlineStr">
         <is>
-          <t>Lahaina — seasonal fresh fruit bowls &amp; dairy-free sorbets</t>
+          <t>Kihei — tropical acai bowl + healthy groceries</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="28" t="inlineStr">
         <is>
-          <t>Leoda's Kitchen &amp; Pie Shop</t>
+          <t>Wow Wow Hawaiian Lemonade</t>
         </is>
       </c>
       <c r="B40" s="25" t="inlineStr">
         <is>
-          <t>820 Olowalu Village Rd — pies, pastries, savory pot pies</t>
+          <t>Kihei — acai bowls + fresh lemonades</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="28" t="inlineStr">
         <is>
+          <t>Maui Fruit Ninja</t>
+        </is>
+      </c>
+      <c r="B41" s="25" t="inlineStr">
+        <is>
+          <t>Lahaina — seasonal fresh fruit bowls &amp; dairy-free sorbets</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="28" t="inlineStr">
+        <is>
+          <t>Leoda's Kitchen &amp; Pie Shop</t>
+        </is>
+      </c>
+      <c r="B42" s="25" t="inlineStr">
+        <is>
+          <t>820 Olowalu Village Rd — pies, pastries, savory pot pies</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="28" t="inlineStr">
+        <is>
           <t>Ahihi-Kinau Marine Preserve</t>
         </is>
       </c>
-      <c r="B41" s="25" t="inlineStr">
+      <c r="B43" s="25" t="inlineStr">
         <is>
           <t>South Maui / La Perouse Bay — tide pools, lava fields</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="21" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="21" t="inlineStr">
         <is>
           <t>🧳 PACKING REMINDERS</t>
-        </is>
-      </c>
-      <c r="B43" s="22" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="25" t="inlineStr">
-        <is>
-          <t>☐ Reef-safe sunscreen (required by Hawaii law)</t>
-        </is>
-      </c>
-      <c r="B44" s="22" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="25" t="inlineStr">
-        <is>
-          <t>☐ Snorkel gear (or rent on island)</t>
         </is>
       </c>
       <c r="B45" s="22" t="n"/>
@@ -3829,7 +3878,7 @@
     <row r="46">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>☐ Comfortable walking shoes</t>
+          <t>☐ Reef-safe sunscreen (required by Hawaii law)</t>
         </is>
       </c>
       <c r="B46" s="22" t="n"/>
@@ -3837,7 +3886,7 @@
     <row r="47">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>☐ Warm layers for Haleakala sunrise (30-40°F at summit)</t>
+          <t>☐ Snorkel gear (or rent on island)</t>
         </is>
       </c>
       <c r="B47" s="22" t="n"/>
@@ -3845,7 +3894,7 @@
     <row r="48">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>☐ Rain jacket (Road to Hana gets wet)</t>
+          <t>☐ Comfortable walking shoes</t>
         </is>
       </c>
       <c r="B48" s="22" t="n"/>
@@ -3853,7 +3902,7 @@
     <row r="49">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>☐ Water shoes (rocky beaches)</t>
+          <t>☐ Warm layers for Haleakala sunrise (30-40°F at summit)</t>
         </is>
       </c>
       <c r="B49" s="22" t="n"/>
@@ -3861,7 +3910,7 @@
     <row r="50">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>☐ Swimsuits &amp; rash guards</t>
+          <t>☐ Rain jacket (Road to Hana gets wet)</t>
         </is>
       </c>
       <c r="B50" s="22" t="n"/>
@@ -3869,7 +3918,7 @@
     <row r="51">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>☐ Reusable water bottles (HYDRATE — extra for pregnancy!)</t>
+          <t>☐ Water shoes (rocky beaches)</t>
         </is>
       </c>
       <c r="B51" s="22" t="n"/>
@@ -3877,7 +3926,7 @@
     <row r="52">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>☐ Portable charger / power bank</t>
+          <t>☐ Swimsuits &amp; rash guards</t>
         </is>
       </c>
       <c r="B52" s="22" t="n"/>
@@ -3885,7 +3934,7 @@
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>☐ Car phone mount for Hana drive</t>
+          <t>☐ Reusable water bottles (HYDRATE — extra for pregnancy!)</t>
         </is>
       </c>
       <c r="B53" s="22" t="n"/>
@@ -3893,7 +3942,7 @@
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>☐ Dramamine (check w/ OB for pregnancy-safe option)</t>
+          <t>☐ Portable charger / power bank</t>
         </is>
       </c>
       <c r="B54" s="22" t="n"/>
@@ -3901,7 +3950,7 @@
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>☐ Dry bag for water activities</t>
+          <t>☐ Car phone mount for Hana drive</t>
         </is>
       </c>
       <c r="B55" s="22" t="n"/>
@@ -3909,7 +3958,7 @@
     <row r="56">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>☐ Compression socks for flights</t>
+          <t>☐ Dramamine (check w/ OB for pregnancy-safe option)</t>
         </is>
       </c>
       <c r="B56" s="22" t="n"/>
@@ -3917,7 +3966,7 @@
     <row r="57">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>☐ Prenatal vitamins &amp; pregnancy meds</t>
+          <t>☐ Dry bag for water activities</t>
         </is>
       </c>
       <c r="B57" s="22" t="n"/>
@@ -3925,7 +3974,7 @@
     <row r="58">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>☐ Pregnancy pillow or support wedge</t>
+          <t>☐ Compression socks for flights</t>
         </is>
       </c>
       <c r="B58" s="22" t="n"/>
@@ -3933,62 +3982,78 @@
     <row r="59">
       <c r="A59" s="25" t="inlineStr">
         <is>
+          <t>☐ Prenatal vitamins &amp; pregnancy meds</t>
+        </is>
+      </c>
+      <c r="B59" s="22" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="25" t="inlineStr">
+        <is>
+          <t>☐ Pregnancy pillow or support wedge</t>
+        </is>
+      </c>
+      <c r="B60" s="22" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="25" t="inlineStr">
+        <is>
           <t>☐ Snacks for Hana (crackers, fruit, nuts)</t>
         </is>
       </c>
-      <c r="B59" s="22" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="21" t="inlineStr">
+      <c r="B61" s="22" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="21" t="inlineStr">
         <is>
           <t>🚨 EMERGENCY CONTACTS</t>
         </is>
       </c>
-      <c r="B61" s="22" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="23" t="inlineStr">
-        <is>
-          <t>Maui Memorial Medical Center</t>
-        </is>
-      </c>
-      <c r="B62" s="24" t="inlineStr">
-        <is>
-          <t>(808) 244-9056</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="23" t="inlineStr">
-        <is>
-          <t>Maui Police (non-emergency)</t>
-        </is>
-      </c>
-      <c r="B63" s="24" t="inlineStr">
-        <is>
-          <t>(808) 244-6400</t>
-        </is>
-      </c>
+      <c r="B63" s="22" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="23" t="inlineStr">
         <is>
-          <t>Hawaii Visitor Emergency Line</t>
+          <t>Maui Memorial Medical Center</t>
         </is>
       </c>
       <c r="B64" s="24" t="inlineStr">
         <is>
-          <t>911</t>
+          <t>(808) 244-9056</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="23" t="inlineStr">
         <is>
+          <t>Maui Police (non-emergency)</t>
+        </is>
+      </c>
+      <c r="B65" s="24" t="inlineStr">
+        <is>
+          <t>(808) 244-6400</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="23" t="inlineStr">
+        <is>
+          <t>Hawaii Visitor Emergency Line</t>
+        </is>
+      </c>
+      <c r="B66" s="24" t="inlineStr">
+        <is>
+          <t>911</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="23" t="inlineStr">
+        <is>
           <t>Poison Control</t>
         </is>
       </c>
-      <c r="B65" s="24" t="inlineStr">
+      <c r="B67" s="24" t="inlineStr">
         <is>
           <t>1-800-222-1222</t>
         </is>
@@ -3997,9 +4062,10 @@
   </sheetData>
   <mergeCells count="33">
     <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A60:B60"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A49:B49"/>
     <mergeCell ref="A51:B51"/>
@@ -4014,29 +4080,28 @@
     <mergeCell ref="A55:B55"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A21:B21"/>
     <mergeCell ref="A57:B57"/>
     <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A32:B32"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A53:B53"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A52:B52"/>
-    <mergeCell ref="A43:B43"/>
     <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A63:B63"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A9:B9"/>
     <mergeCell ref="A58:B58"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Cafe O'Lei Kihei (must-do) to Day 5 relaxation day
- Steps from the Airbnb at 2439 S Kihei Rd
- Old Lahaina Luau already included as must-book on Day 7

Co-Authored-By: Claude (claude-opus-4-6[1m]) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/maui_itinerary.xlsx
+++ b/maui_itinerary.xlsx
@@ -853,7 +853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2397,12 +2397,12 @@
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>Shave ice at Surfing Monkey Shave Ice</t>
+          <t>Lunch at Cafe O'Lei Kihei</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>1881 S Kihei Rd, Kihei</t>
+          <t>2439 S Kihei Rd #201A, Kihei</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
@@ -2413,92 +2413,92 @@
       <c r="G37" s="8" t="inlineStr"/>
       <c r="H37" s="8" t="inlineStr">
         <is>
+          <t>Must-do! Steps from the Airbnb. Great local spot</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Mon, May 4</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>2:00 PM</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Shave ice at Surfing Monkey Shave Ice</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>1881 S Kihei Rd, Kihei</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>Food / Dining</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr"/>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
           <t>Kona coffee flavor + vegan coconut milk ice cream option</t>
         </is>
       </c>
-      <c r="I37" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="10" t="n">
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
         <is>
           <t>Mon, May 4</t>
         </is>
       </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>2:00 – 4:00 PM</t>
-        </is>
-      </c>
-      <c r="D38" s="11" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>2:30 – 4:00 PM</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
         <is>
           <t>Prenatal spa treatment or continued beach time</t>
         </is>
       </c>
-      <c r="E38" s="11" t="inlineStr">
+      <c r="E39" s="11" t="inlineStr">
         <is>
           <t>Wailea / Kihei</t>
         </is>
       </c>
-      <c r="F38" s="10" t="inlineStr">
+      <c r="F39" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G38" s="11" t="inlineStr"/>
-      <c r="H38" s="11" t="inlineStr">
+      <c r="G39" s="11" t="inlineStr"/>
+      <c r="H39" s="11" t="inlineStr">
         <is>
           <t>Prenatal massage at a Wailea spa — Brittany's choice!</t>
         </is>
       </c>
-      <c r="I38" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>Mon, May 4</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>4:15 PM</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Fresh fruit &amp; acai at Hawaiian Moons Natural Foods</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>Kihei</t>
-        </is>
-      </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Food / Dining</t>
-        </is>
-      </c>
-      <c r="G39" s="8" t="inlineStr"/>
-      <c r="H39" s="8" t="inlineStr">
-        <is>
-          <t>Tropical acai bowl + stock up on healthy snacks</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="inlineStr">
+      <c r="I39" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2515,125 +2515,121 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
+          <t>4:15 PM</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Fresh fruit &amp; acai at Hawaiian Moons Natural Foods</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Kihei</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>Food / Dining</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr"/>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>Tropical acai bowl + stock up on healthy snacks</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Mon, May 4</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="D40" s="8" t="inlineStr">
+      <c r="D41" s="8" t="inlineStr">
         <is>
           <t>Dinner at Monkeypod Kitchen (happy hour, live music)</t>
         </is>
       </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="E41" s="8" t="inlineStr">
         <is>
           <t>Wailea</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr">
+      <c r="F41" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G40" s="9" t="inlineStr">
+      <c r="G41" s="9" t="inlineStr">
         <is>
           <t>Monkeypod Kitchen</t>
         </is>
       </c>
-      <c r="H40" s="8" t="inlineStr">
+      <c r="H41" s="8" t="inlineStr">
         <is>
           <t>Great mocktails for Brittany!</t>
         </is>
       </c>
-      <c r="I40" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="15" t="n">
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B41" s="15" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C41" s="15" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
         <is>
           <t>6:00 AM</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr">
+      <c r="D42" s="16" t="inlineStr">
         <is>
           <t>Molokini Crater snorkel boat tour (departs Ma'alaea)</t>
         </is>
       </c>
-      <c r="E41" s="16" t="inlineStr">
+      <c r="E42" s="16" t="inlineStr">
         <is>
           <t>Ma'alaea Harbor</t>
         </is>
       </c>
-      <c r="F41" s="15" t="inlineStr">
+      <c r="F42" s="15" t="inlineStr">
         <is>
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G41" s="17" t="inlineStr">
+      <c r="G42" s="17" t="inlineStr">
         <is>
           <t>Pacific Whale Foundation</t>
         </is>
       </c>
-      <c r="H41" s="16" t="inlineStr">
+      <c r="H42" s="16" t="inlineStr">
         <is>
           <t>⚠️ BOOK IN ADVANCE. Bring Dramamine (check w/ OB)</t>
         </is>
       </c>
-      <c r="I41" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>Tue, May 5</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>11:30 AM</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>Lunch at Coconut's Fish Cafe</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>Kihei</t>
-        </is>
-      </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>Food / Dining</t>
-        </is>
-      </c>
-      <c r="G42" s="9" t="inlineStr">
-        <is>
-          <t>Coconut's Fish Cafe</t>
-        </is>
-      </c>
-      <c r="H42" s="8" t="inlineStr">
-        <is>
-          <t>Cooked fish tacos — pregnancy safe</t>
-        </is>
-      </c>
-      <c r="I42" s="7" t="inlineStr">
+      <c r="I42" s="15" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2650,412 +2646,416 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
+          <t>11:30 AM</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Lunch at Coconut's Fish Cafe</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Kihei</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>Food / Dining</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>Coconut's Fish Cafe</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>Cooked fish tacos — pregnancy safe</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Tue, May 5</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
           <t>12:15 PM</t>
         </is>
       </c>
-      <c r="D43" s="8" t="inlineStr">
+      <c r="D44" s="8" t="inlineStr">
         <is>
           <t>Shave ice at Peace Love Shave Ice</t>
         </is>
       </c>
-      <c r="E43" s="8" t="inlineStr">
+      <c r="E44" s="8" t="inlineStr">
         <is>
           <t>Azeka Plaza, Kihei</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G43" s="8" t="inlineStr"/>
-      <c r="H43" s="8" t="inlineStr">
+      <c r="G44" s="8" t="inlineStr"/>
+      <c r="H44" s="8" t="inlineStr">
         <is>
           <t>Organic syrups, Thai Iced Tea flavor, Roselani ice cream base</t>
         </is>
       </c>
-      <c r="I43" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="18" t="n">
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="B44" s="18" t="inlineStr">
+      <c r="B45" s="18" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C44" s="18" t="inlineStr">
+      <c r="C45" s="18" t="inlineStr">
         <is>
           <t>1:00 PM</t>
         </is>
       </c>
-      <c r="D44" s="19" t="inlineStr">
+      <c r="D45" s="19" t="inlineStr">
         <is>
           <t>Visit Ahihi-Kinau Marine Preserve — tide pools &amp; lava fields</t>
         </is>
       </c>
-      <c r="E44" s="19" t="inlineStr">
+      <c r="E45" s="19" t="inlineStr">
         <is>
           <t>Wailea / La Perouse Bay</t>
         </is>
       </c>
-      <c r="F44" s="18" t="inlineStr">
+      <c r="F45" s="18" t="inlineStr">
         <is>
           <t>Nature / Hiking</t>
         </is>
       </c>
-      <c r="G44" s="19" t="inlineStr"/>
-      <c r="H44" s="19" t="inlineStr">
+      <c r="G45" s="19" t="inlineStr"/>
+      <c r="H45" s="19" t="inlineStr">
         <is>
           <t>Beautiful natural reserve. Gentle exploring, tide pools</t>
         </is>
       </c>
-      <c r="I44" s="18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="10" t="n">
+      <c r="I45" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B45" s="10" t="inlineStr">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C45" s="10" t="inlineStr">
+      <c r="C46" s="10" t="inlineStr">
         <is>
           <t>2:30 – 4:30 PM</t>
         </is>
       </c>
-      <c r="D45" s="11" t="inlineStr">
+      <c r="D46" s="11" t="inlineStr">
         <is>
           <t>Beach relaxation at Big Beach (Makena State Park)</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Makena</t>
         </is>
       </c>
-      <c r="F45" s="10" t="inlineStr">
+      <c r="F46" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G45" s="11" t="inlineStr"/>
-      <c r="H45" s="11" t="inlineStr">
+      <c r="G46" s="11" t="inlineStr"/>
+      <c r="H46" s="11" t="inlineStr">
         <is>
           <t>Watch the bodyboarders! Brittany should wade gently — big shore break</t>
         </is>
       </c>
-      <c r="I45" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="15" t="n">
+      <c r="I46" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B46" s="15" t="inlineStr">
+      <c r="B47" s="15" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C46" s="15" t="inlineStr">
+      <c r="C47" s="15" t="inlineStr">
         <is>
           <t>6:00 PM</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
+      <c r="D47" s="16" t="inlineStr">
         <is>
           <t>Dinner at Mama's Fish House</t>
         </is>
       </c>
-      <c r="E46" s="16" t="inlineStr">
+      <c r="E47" s="16" t="inlineStr">
         <is>
           <t>Pa'ia</t>
         </is>
       </c>
-      <c r="F46" s="15" t="inlineStr">
+      <c r="F47" s="15" t="inlineStr">
         <is>
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G46" s="17" t="inlineStr">
+      <c r="G47" s="17" t="inlineStr">
         <is>
           <t>Mama's Fish House</t>
         </is>
       </c>
-      <c r="H46" s="16" t="inlineStr">
+      <c r="H47" s="16" t="inlineStr">
         <is>
           <t>⚠️ RESERVE WELL IN ADVANCE. Order cooked dishes for Brittany</t>
         </is>
       </c>
-      <c r="I46" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="18" t="n">
+      <c r="I47" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="B47" s="18" t="inlineStr">
+      <c r="B48" s="18" t="inlineStr">
         <is>
           <t>Wed, May 6</t>
         </is>
       </c>
-      <c r="C47" s="18" t="inlineStr">
+      <c r="C48" s="18" t="inlineStr">
         <is>
           <t>8:30 AM</t>
         </is>
       </c>
-      <c r="D47" s="19" t="inlineStr">
+      <c r="D48" s="19" t="inlineStr">
         <is>
           <t>'Iao Valley State Monument — 'Iao Needle viewpoint walk</t>
         </is>
       </c>
-      <c r="E47" s="19" t="inlineStr">
+      <c r="E48" s="19" t="inlineStr">
         <is>
           <t>'Iao Valley</t>
         </is>
       </c>
-      <c r="F47" s="18" t="inlineStr">
+      <c r="F48" s="18" t="inlineStr">
         <is>
           <t>Nature / Hiking</t>
         </is>
       </c>
-      <c r="G47" s="20" t="inlineStr">
+      <c r="G48" s="20" t="inlineStr">
         <is>
           <t>'Iao Valley Info</t>
         </is>
       </c>
-      <c r="H47" s="19" t="inlineStr">
+      <c r="H48" s="19" t="inlineStr">
         <is>
           <t>Short paved path. Perfect for pregnancy</t>
         </is>
       </c>
-      <c r="I47" s="18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="7" t="n">
+      <c r="I48" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B49" s="7" t="inlineStr">
         <is>
           <t>Wed, May 6</t>
         </is>
       </c>
-      <c r="C48" s="7" t="inlineStr">
+      <c r="C49" s="7" t="inlineStr">
         <is>
           <t>10:30 AM</t>
         </is>
       </c>
-      <c r="D48" s="8" t="inlineStr">
+      <c r="D49" s="8" t="inlineStr">
         <is>
           <t>Lunch at Sam Sato's (dry mein and manju)</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
+      <c r="E49" s="8" t="inlineStr">
         <is>
           <t>Wailuku</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F49" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G48" s="8" t="inlineStr"/>
-      <c r="H48" s="8" t="inlineStr">
+      <c r="G49" s="8" t="inlineStr"/>
+      <c r="H49" s="8" t="inlineStr">
         <is>
           <t>Famous local spot — the manju is a must!</t>
         </is>
       </c>
-      <c r="I48" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="10" t="n">
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B49" s="10" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>Wed, May 6</t>
         </is>
       </c>
-      <c r="C49" s="10" t="inlineStr">
+      <c r="C50" s="10" t="inlineStr">
         <is>
           <t>12:00 – 4:00 PM</t>
         </is>
       </c>
-      <c r="D49" s="11" t="inlineStr">
+      <c r="D50" s="11" t="inlineStr">
         <is>
           <t>Beach relaxation or Wailea Beach Path walk</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Wailea / Kihei</t>
         </is>
       </c>
-      <c r="F49" s="10" t="inlineStr">
+      <c r="F50" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G49" s="11" t="inlineStr"/>
-      <c r="H49" s="11" t="inlineStr">
+      <c r="G50" s="11" t="inlineStr"/>
+      <c r="H50" s="11" t="inlineStr">
         <is>
           <t>Flat oceanfront path or lazy afternoon at the beach</t>
         </is>
       </c>
-      <c r="I49" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="15" t="n">
+      <c r="I50" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="B50" s="15" t="inlineStr">
+      <c r="B51" s="15" t="inlineStr">
         <is>
           <t>Wed, May 6</t>
         </is>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr">
         <is>
           <t>5:00 PM</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="D51" s="16" t="inlineStr">
         <is>
           <t>Luau — Old Lahaina Luau or Feast at Lele</t>
         </is>
       </c>
-      <c r="E50" s="16" t="inlineStr">
+      <c r="E51" s="16" t="inlineStr">
         <is>
           <t>Lahaina</t>
         </is>
       </c>
-      <c r="F50" s="15" t="inlineStr">
+      <c r="F51" s="15" t="inlineStr">
         <is>
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G50" s="17" t="inlineStr">
+      <c r="G51" s="17" t="inlineStr">
         <is>
           <t>Old Lahaina Luau</t>
         </is>
       </c>
-      <c r="H50" s="16" t="inlineStr">
+      <c r="H51" s="16" t="inlineStr">
         <is>
           <t>⚠️ BOOK IN ADVANCE. Seated &amp; relaxed — perfect for pregnancy</t>
         </is>
       </c>
-      <c r="I50" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="10" t="n">
+      <c r="I51" s="15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B51" s="10" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>Thu, May 7</t>
         </is>
       </c>
-      <c r="C51" s="10" t="inlineStr">
+      <c r="C52" s="10" t="inlineStr">
         <is>
           <t>8:00 AM</t>
         </is>
       </c>
-      <c r="D51" s="11" t="inlineStr">
+      <c r="D52" s="11" t="inlineStr">
         <is>
           <t>Easy morning walk along Wailea Beach Path</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Wailea</t>
         </is>
       </c>
-      <c r="F51" s="10" t="inlineStr">
+      <c r="F52" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G51" s="11" t="inlineStr"/>
-      <c r="H51" s="11" t="inlineStr">
+      <c r="G52" s="11" t="inlineStr"/>
+      <c r="H52" s="11" t="inlineStr">
         <is>
           <t>Flat oceanfront path, gorgeous views. Great gentle exercise</t>
         </is>
       </c>
-      <c r="I51" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B52" s="7" t="inlineStr">
-        <is>
-          <t>Thu, May 7</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="inlineStr">
-        <is>
-          <t>9:00 AM</t>
-        </is>
-      </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>Acai bowl at Brekkie Bowls food truck</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>Wailea</t>
-        </is>
-      </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>Food / Dining</t>
-        </is>
-      </c>
-      <c r="G52" s="8" t="inlineStr"/>
-      <c r="H52" s="8" t="inlineStr">
-        <is>
-          <t>Superfood acai bowl — perfect pregnancy fuel!</t>
-        </is>
-      </c>
-      <c r="I52" s="7" t="inlineStr">
+      <c r="I52" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3072,17 +3072,17 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>10:30 AM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>Shave ice at Ululani's (Kihei location)</t>
+          <t>Acai bowl at Brekkie Bowls food truck</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>61 S Kihei Rd, Kihei</t>
+          <t>Wailea</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
@@ -3090,14 +3090,10 @@
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G53" s="9" t="inlineStr">
-        <is>
-          <t>Ululani's</t>
-        </is>
-      </c>
+      <c r="G53" s="8" t="inlineStr"/>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>Round 2! Try a different flavor combo</t>
+          <t>Superfood acai bowl — perfect pregnancy fuel!</t>
         </is>
       </c>
       <c r="I53" s="7" t="inlineStr">
@@ -3117,244 +3113,248 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
+          <t>10:30 AM</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Shave ice at Ululani's (Kihei location)</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>61 S Kihei Rd, Kihei</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>Food / Dining</t>
+        </is>
+      </c>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>Ululani's</t>
+        </is>
+      </c>
+      <c r="H54" s="8" t="inlineStr">
+        <is>
+          <t>Round 2! Try a different flavor combo</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Thu, May 7</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
           <t>11:15 AM</t>
         </is>
       </c>
-      <c r="D54" s="8" t="inlineStr">
+      <c r="D55" s="8" t="inlineStr">
         <is>
           <t>Fresh fruit bowls at Maui Fruit Ninja</t>
         </is>
       </c>
-      <c r="E54" s="8" t="inlineStr">
+      <c r="E55" s="8" t="inlineStr">
         <is>
           <t>Lahaina</t>
         </is>
       </c>
-      <c r="F54" s="7" t="inlineStr">
+      <c r="F55" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G54" s="9" t="inlineStr">
+      <c r="G55" s="9" t="inlineStr">
         <is>
           <t>Maui Fruit Ninja</t>
         </is>
       </c>
-      <c r="H54" s="8" t="inlineStr">
+      <c r="H55" s="8" t="inlineStr">
         <is>
           <t>Seasonal tropical fruit bowls &amp; dairy-free sorbets</t>
         </is>
       </c>
-      <c r="I54" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="10" t="n">
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="B55" s="10" t="inlineStr">
+      <c r="B56" s="10" t="inlineStr">
         <is>
           <t>Thu, May 7</t>
         </is>
       </c>
-      <c r="C55" s="10" t="inlineStr">
+      <c r="C56" s="10" t="inlineStr">
         <is>
           <t>12:30 – 3:00 PM</t>
         </is>
       </c>
-      <c r="D55" s="11" t="inlineStr">
+      <c r="D56" s="11" t="inlineStr">
         <is>
           <t>Beach time + revisits, shopping, souvenirs</t>
         </is>
       </c>
-      <c r="E55" s="11" t="inlineStr">
+      <c r="E56" s="11" t="inlineStr">
         <is>
           <t>Various / Kihei</t>
         </is>
       </c>
-      <c r="F55" s="10" t="inlineStr">
+      <c r="F56" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G55" s="11" t="inlineStr"/>
-      <c r="H55" s="11" t="inlineStr">
+      <c r="G56" s="11" t="inlineStr"/>
+      <c r="H56" s="11" t="inlineStr">
         <is>
           <t>Last full beach day! Soak it in</t>
         </is>
       </c>
-      <c r="I55" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="7" t="n">
+      <c r="I56" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="B57" s="7" t="inlineStr">
         <is>
           <t>Thu, May 7</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>3:30 PM</t>
         </is>
       </c>
-      <c r="D56" s="8" t="inlineStr">
+      <c r="D57" s="8" t="inlineStr">
         <is>
           <t>Pie &amp; treats at Leoda's Kitchen and Pie Shop</t>
         </is>
       </c>
-      <c r="E56" s="8" t="inlineStr">
+      <c r="E57" s="8" t="inlineStr">
         <is>
           <t>820 Olowalu Village Rd, Lahaina</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F57" s="7" t="inlineStr">
         <is>
           <t>Food / Dining</t>
         </is>
       </c>
-      <c r="G56" s="8" t="inlineStr"/>
-      <c r="H56" s="8" t="inlineStr">
+      <c r="G57" s="8" t="inlineStr"/>
+      <c r="H57" s="8" t="inlineStr">
         <is>
           <t>Famous pies — banana cream, macnut, savory pot pies</t>
         </is>
       </c>
-      <c r="I56" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="15" t="n">
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B57" s="15" t="inlineStr">
+      <c r="B58" s="15" t="inlineStr">
         <is>
           <t>Thu, May 7</t>
         </is>
       </c>
-      <c r="C57" s="15" t="inlineStr">
+      <c r="C58" s="15" t="inlineStr">
         <is>
           <t>5:30 PM</t>
         </is>
       </c>
-      <c r="D57" s="16" t="inlineStr">
+      <c r="D58" s="16" t="inlineStr">
         <is>
           <t>Final sunset dinner at Merriman's Kapalua</t>
         </is>
       </c>
-      <c r="E57" s="16" t="inlineStr">
+      <c r="E58" s="16" t="inlineStr">
         <is>
           <t>Kapalua</t>
         </is>
       </c>
-      <c r="F57" s="15" t="inlineStr">
+      <c r="F58" s="15" t="inlineStr">
         <is>
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G57" s="17" t="inlineStr">
+      <c r="G58" s="17" t="inlineStr">
         <is>
           <t>Merriman's Kapalua</t>
         </is>
       </c>
-      <c r="H57" s="16" t="inlineStr">
+      <c r="H58" s="16" t="inlineStr">
         <is>
           <t>BOOKED — hoping for outdoor 5:30 seating (waitlisted). Keep checking!</t>
         </is>
       </c>
-      <c r="I57" s="15" t="inlineStr">
+      <c r="I58" s="15" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="10" t="n">
+    <row r="59">
+      <c r="A59" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="B58" s="10" t="inlineStr">
+      <c r="B59" s="10" t="inlineStr">
         <is>
           <t>Fri, May 8</t>
         </is>
       </c>
-      <c r="C58" s="10" t="inlineStr">
+      <c r="C59" s="10" t="inlineStr">
         <is>
           <t>7:00 AM</t>
         </is>
       </c>
-      <c r="D58" s="11" t="inlineStr">
+      <c r="D59" s="11" t="inlineStr">
         <is>
           <t>Last morning beach walk at Kamaole Beach</t>
         </is>
       </c>
-      <c r="E58" s="11" t="inlineStr">
+      <c r="E59" s="11" t="inlineStr">
         <is>
           <t>Kihei</t>
         </is>
       </c>
-      <c r="F58" s="10" t="inlineStr">
+      <c r="F59" s="10" t="inlineStr">
         <is>
           <t>Beach / Water</t>
         </is>
       </c>
-      <c r="G58" s="11" t="inlineStr"/>
-      <c r="H58" s="11" t="inlineStr">
+      <c r="G59" s="11" t="inlineStr"/>
+      <c r="H59" s="11" t="inlineStr">
         <is>
           <t>One last Maui sunrise moment</t>
         </is>
       </c>
-      <c r="I58" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>Fri, May 8</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>8:00 – 10:00 AM</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Pack up &amp; check out of Airbnb by 11 AM. Return rental car.</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>2777 S Kihei Rd → OGG</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>Logistics</t>
-        </is>
-      </c>
-      <c r="G59" s="5" t="inlineStr"/>
-      <c r="H59" s="5" t="inlineStr">
-        <is>
-          <t>Airbnb check-out: 11:00 AM. Airport is ~25 min from Kihei</t>
-        </is>
-      </c>
-      <c r="I59" s="4" t="inlineStr">
+      <c r="I59" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3371,27 +3371,68 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
+          <t>8:00 – 10:00 AM</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Pack up &amp; check out of Airbnb by 11 AM. Return rental car.</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>2777 S Kihei Rd → OGG</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr"/>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>Airbnb check-out: 11:00 AM. Airport is ~25 min from Kihei</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Fri, May 8</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
           <t>10:40 AM</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>Flight AS 978 OGG → SFO. Arrive 6:44 PM.</t>
         </is>
       </c>
-      <c r="E60" s="5" t="inlineStr">
+      <c r="E61" s="5" t="inlineStr">
         <is>
           <t>OGG Airport</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr">
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t>Logistics</t>
         </is>
       </c>
-      <c r="G60" s="5" t="inlineStr"/>
-      <c r="H60" s="5" t="inlineStr"/>
-      <c r="I60" s="4" t="inlineStr">
+      <c r="G61" s="5" t="inlineStr"/>
+      <c r="H61" s="5" t="inlineStr"/>
+      <c r="I61" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>

<commit_message>
Update reservations: Mama's 12PM, Luau 5:45PM Tue, Sunset Sail 5PM Wed, Wai'anapanapa 12:30-3PM
- Mama's Fish House: RESERVED Tue May 5 at 12:00 PM (moved to lunch)
- Old Lahaina Luau: RESERVED Tue May 5 at 5:45 PM (moved from Wed to Tue)
- Ka'anapali Sunset Sail: RESERVED Wed May 6 at 5:00 PM (new, Sheraton departure)
- Wai'anapanapa: RESERVED 12:30-3:00 PM window, must leave by 3 PM
- Day 6 reworked: Molokini AM + Mama's lunch + Luau evening
- Day 7 reworked: 'Iao Valley + Ahihi-Kinau + Sunset Sail
- Full spreadsheet rebuild to match HTML

Co-Authored-By: Claude (claude-opus-4-6[1m]) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/maui_itinerary.xlsx
+++ b/maui_itinerary.xlsx
@@ -186,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -261,6 +261,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -945,7 +946,7 @@
       </c>
       <c r="G2" s="6" t="inlineStr">
         <is>
-          <t>Costco Travel Rental Cars</t>
+          <t>Costco Travel</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
@@ -975,7 +976,7 @@
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Lunch at Tin Roof Maui (Sheldon Simeon's spot)</t>
+          <t>Lunch at Tin Roof Maui</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
@@ -985,7 +986,7 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
@@ -995,7 +996,7 @@
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Try garlic noodles! Avoid raw ahi (pregnancy)</t>
+          <t>Avoid raw ahi (pregnancy)</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
@@ -1030,13 +1031,13 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr"/>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Great post-flight snack — fresh fruit &amp; acai</t>
+          <t>Great post-flight snack</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
@@ -1071,13 +1072,13 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G5" s="11" t="inlineStr"/>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>Airbnb check-in not until 4 PM — hit the beach first! Drop bags at car</t>
+          <t>Airbnb check-in not until 4 PM — hit the beach first!</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr">
@@ -1190,7 +1191,7 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -1200,7 +1201,7 @@
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Order cooked fish (avoid raw/sushi for pregnancy)</t>
+          <t>Order cooked fish (pregnancy)</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
@@ -1225,7 +1226,7 @@
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Gentle snorkel at Napili Bay (turtles, calm water)</t>
+          <t>Gentle snorkel at Napili Bay</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -1235,13 +1236,13 @@
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr"/>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>Snorkeling OK if Brittany comfortable — no scuba</t>
+          <t>Snorkeling OK if Brittany comfortable</t>
         </is>
       </c>
       <c r="I9" s="10" t="inlineStr">
@@ -1276,13 +1277,13 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr"/>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>Float, enjoy the turtles. Shade &amp; hydration for Brittany</t>
+          <t>Shade &amp; hydration for Brittany</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
@@ -1317,13 +1318,13 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr"/>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>Get cooked options for Brittany (no raw ahi)</t>
+          <t>Get cooked options for Brittany</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
@@ -1348,7 +1349,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Shave ice at Ululani's Hawaiian Shave Ice</t>
+          <t>Shave ice at Ululani's</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -1358,7 +1359,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -1368,7 +1369,7 @@
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>Get ice cream base — Roselani macadamia nut!</t>
+          <t>Roselani macadamia nut ice cream base!</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
@@ -1393,7 +1394,7 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Explore Lahaina town — banyan tree, Front St, galleries</t>
+          <t>Explore Lahaina town</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
@@ -1403,7 +1404,7 @@
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Cultural / Sightseeing</t>
+          <t>Cultural</t>
         </is>
       </c>
       <c r="G13" s="14" t="inlineStr">
@@ -1413,7 +1414,7 @@
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Easy walking. Be respectful of rebuilding efforts</t>
+          <t>Easy walking. Be respectful of rebuilding</t>
         </is>
       </c>
       <c r="I13" s="12" t="inlineStr">
@@ -1448,7 +1449,7 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -1456,11 +1457,7 @@
           <t>Mala Ocean Tavern</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
-        <is>
-          <t>Alt: Fleetwood's on Front St if reopened</t>
-        </is>
-      </c>
+      <c r="H14" s="8" t="inlineStr"/>
       <c r="I14" s="7" t="inlineStr">
         <is>
           <t>N</t>
@@ -1483,7 +1480,7 @@
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>Depart for Haleakala summit (~1.5–2 hr drive)</t>
+          <t>Depart for Haleakala summit</t>
         </is>
       </c>
       <c r="E15" s="16" t="inlineStr">
@@ -1498,7 +1495,7 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>Recreation.gov Reservations</t>
+          <t>Recreation.gov</t>
         </is>
       </c>
       <c r="H15" s="16" t="inlineStr">
@@ -1544,7 +1541,7 @@
       <c r="G16" s="16" t="inlineStr"/>
       <c r="H16" s="16" t="inlineStr">
         <is>
-          <t>Limit to ~30 min at summit — thin air &amp; pregnancy. Leave if dizzy</t>
+          <t>Limit to ~30 min — thin air &amp; pregnancy</t>
         </is>
       </c>
       <c r="I16" s="15" t="inlineStr">
@@ -1569,7 +1566,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Drive Upcountry. Visit Ali'i Kula Lavender Farm.</t>
+          <t>Ali'i Kula Lavender Farm</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -1579,7 +1576,7 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Nature / Hiking</t>
+          <t>Nature/Hiking</t>
         </is>
       </c>
       <c r="G17" s="20" t="inlineStr">
@@ -1624,7 +1621,7 @@
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr"/>
@@ -1651,7 +1648,7 @@
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>Surfing Goat Dairy or MauiWine at Ulupalakua</t>
+          <t>Surfing Goat Dairy or MauiWine</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -1661,7 +1658,7 @@
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Cultural / Sightseeing</t>
+          <t>Cultural</t>
         </is>
       </c>
       <c r="G19" s="14" t="inlineStr">
@@ -1671,7 +1668,7 @@
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>Non-alcoholic tastings for Brittany. Goat dairy is fun!</t>
+          <t>Non-alcoholic tastings for Brittany</t>
         </is>
       </c>
       <c r="I19" s="12" t="inlineStr">
@@ -1696,23 +1693,23 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Stop at Leoda's Kitchen &amp; Pie Shop on drive back</t>
+          <t>Leoda's Kitchen &amp; Pie Shop</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>820 Olowalu Village Rd, Lahaina</t>
+          <t>820 Olowalu Village Rd</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr"/>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>Famous pies — banana cream, macnut, savory pot pies</t>
+          <t>Famous pies — banana cream, macnut</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
@@ -1737,7 +1734,7 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Nap / rest at Airbnb (early wake-up recovery!)</t>
+          <t>Nap / rest at Airbnb</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -1747,7 +1744,7 @@
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr"/>
@@ -1778,7 +1775,7 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Easy dinner — pick up food &amp; eat at Airbnb</t>
+          <t>Easy dinner at Airbnb</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -1788,13 +1785,13 @@
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr"/>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>Rest up for Road to Hana tomorrow</t>
+          <t>Rest up for Hana tomorrow</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
@@ -1812,10 +1809,14 @@
           <t>Sun, May 3</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Night Before</t>
+        </is>
+      </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>📱 APPS: Download Shaka Guide ($) or GyPSy Guide/GuideAlong ($)</t>
+          <t>📱 Download audio tour app (needs wifi!)</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr"/>
@@ -1831,7 +1832,7 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>GPS audio tour — plays automatically as you drive. Works offline! Download night before</t>
+          <t>Works offline! Alt: GyPSy Guide (~$10)</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
@@ -1856,7 +1857,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Depart for Road to Hana. Pack snacks &amp; water!</t>
+          <t>Depart for Road to Hana</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1872,7 +1873,7 @@
       <c r="G24" s="5" t="inlineStr"/>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Start audio tour. Bring crackers, fruit, water for nausea</t>
+          <t>Bring crackers, fruit, water for nausea</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -1897,7 +1898,7 @@
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Twin Falls (Mile 2) — easy short walk</t>
+          <t>Twin Falls (Mile 2)</t>
         </is>
       </c>
       <c r="E25" s="19" t="inlineStr">
@@ -1907,7 +1908,7 @@
       </c>
       <c r="F25" s="18" t="inlineStr">
         <is>
-          <t>Nature / Hiking</t>
+          <t>Nature/Hiking</t>
         </is>
       </c>
       <c r="G25" s="19" t="inlineStr"/>
@@ -1938,7 +1939,7 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Banana bread &amp; fruit smoothie at Halfway to Hana</t>
+          <t>Banana bread &amp; smoothie at Halfway to Hana</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -1948,7 +1949,7 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr"/>
@@ -1989,7 +1990,7 @@
       </c>
       <c r="F27" s="18" t="inlineStr">
         <is>
-          <t>Nature / Hiking</t>
+          <t>Nature/Hiking</t>
         </is>
       </c>
       <c r="G27" s="20" t="inlineStr">
@@ -1999,7 +2000,7 @@
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>Flat walking paths — pregnancy friendly</t>
+          <t>Flat paths — pregnancy friendly</t>
         </is>
       </c>
       <c r="I27" s="18" t="inlineStr">
@@ -2024,7 +2025,7 @@
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Ke'anae Peninsula (Mile 16.5) — scenic viewpoint</t>
+          <t>Ke'anae Peninsula (Mile 16.5)</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -2034,13 +2035,13 @@
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>Cultural / Sightseeing</t>
+          <t>Cultural</t>
         </is>
       </c>
       <c r="G28" s="13" t="inlineStr"/>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>Quick stop, beautiful views, no hiking needed</t>
+          <t>Quick stop, no hiking needed</t>
         </is>
       </c>
       <c r="I28" s="12" t="inlineStr">
@@ -2065,7 +2066,7 @@
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Upper Waikani Falls / Three Bears Falls (Mile 19)</t>
+          <t>Upper Waikani Falls (Mile 19)</t>
         </is>
       </c>
       <c r="E29" s="19" t="inlineStr">
@@ -2075,13 +2076,13 @@
       </c>
       <c r="F29" s="18" t="inlineStr">
         <is>
-          <t>Nature / Hiking</t>
+          <t>Nature/Hiking</t>
         </is>
       </c>
       <c r="G29" s="19" t="inlineStr"/>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>Viewable from the road / short walk</t>
+          <t>Viewable from road</t>
         </is>
       </c>
       <c r="I29" s="18" t="inlineStr">
@@ -2106,7 +2107,7 @@
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>Wai'anapanapa State Park — black sand beach, sea caves</t>
+          <t>Wai'anapanapa State Park — black sand beach</t>
         </is>
       </c>
       <c r="E30" s="16" t="inlineStr">
@@ -2121,17 +2122,17 @@
       </c>
       <c r="G30" s="17" t="inlineStr">
         <is>
-          <t>Wai'anapanapa Reservations</t>
+          <t>Reserve Entry</t>
         </is>
       </c>
       <c r="H30" s="16" t="inlineStr">
         <is>
-          <t>⚠️ MUST RESERVE park entry. Turnaround point</t>
+          <t>✅ RESERVED 12:30–3:00 PM window. Must leave by 3 PM</t>
         </is>
       </c>
       <c r="I30" s="15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2152,7 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Lunch at Braddah Hutts BBQ food truck</t>
+          <t>Lunch at Braddah Hutts BBQ</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -2161,7 +2162,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr"/>
@@ -2192,7 +2193,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Drive back (reverse route — familiar road is easier)</t>
+          <t>Drive back (reverse route)</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -2208,7 +2209,7 @@
       <c r="G32" s="5" t="inlineStr"/>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>Take it slow, stop at missed spots. Brittany can rest/nap</t>
+          <t>Take it slow, Brittany can rest/nap</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -2233,7 +2234,7 @@
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>Arrive back. Easy dinner at Airbnb or Nuka</t>
+          <t>Easy dinner at Airbnb or Nuka</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -2243,13 +2244,13 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G33" s="8" t="inlineStr"/>
       <c r="H33" s="8" t="inlineStr">
         <is>
-          <t>Low-key after a long drive day</t>
+          <t>Low-key after long drive day</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
@@ -2274,7 +2275,7 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Sleep in! Lazy morning at the Airbnb</t>
+          <t>Sleep in! Lazy morning</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
@@ -2284,13 +2285,13 @@
       </c>
       <c r="F34" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G34" s="11" t="inlineStr"/>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>You earned it after Hana. No alarm</t>
+          <t>No alarm</t>
         </is>
       </c>
       <c r="I34" s="10" t="inlineStr">
@@ -2325,13 +2326,13 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G35" s="8" t="inlineStr"/>
       <c r="H35" s="8" t="inlineStr">
         <is>
-          <t>Fresh lemonades + acai bowls. Great healthy breakfast</t>
+          <t>Fresh lemonades + acai bowls</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
@@ -2366,13 +2367,13 @@
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G36" s="11" t="inlineStr"/>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>Walk from Airbnb. Calm water, lifeguards, shade trees</t>
+          <t>Walk from Airbnb. Calm water, lifeguards</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
@@ -2402,18 +2403,18 @@
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>2439 S Kihei Rd #201A, Kihei</t>
+          <t>2439 S Kihei Rd #201A</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G37" s="8" t="inlineStr"/>
       <c r="H37" s="8" t="inlineStr">
         <is>
-          <t>Must-do! Steps from the Airbnb. Great local spot</t>
+          <t>Must-do! Steps from Airbnb</t>
         </is>
       </c>
       <c r="I37" s="7" t="inlineStr">
@@ -2438,23 +2439,23 @@
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>Shave ice at Surfing Monkey Shave Ice</t>
+          <t>Shave ice at Surfing Monkey</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>1881 S Kihei Rd, Kihei</t>
+          <t>1881 S Kihei Rd</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G38" s="8" t="inlineStr"/>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>Kona coffee flavor + vegan coconut milk ice cream option</t>
+          <t>Kona coffee flavor</t>
         </is>
       </c>
       <c r="I38" s="7" t="inlineStr">
@@ -2479,7 +2480,7 @@
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Prenatal spa treatment or continued beach time</t>
+          <t>Prenatal spa or beach time</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
@@ -2489,13 +2490,13 @@
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G39" s="11" t="inlineStr"/>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>Prenatal massage at a Wailea spa — Brittany's choice!</t>
+          <t>Brittany's choice!</t>
         </is>
       </c>
       <c r="I39" s="10" t="inlineStr">
@@ -2520,7 +2521,7 @@
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>Fresh fruit &amp; acai at Hawaiian Moons Natural Foods</t>
+          <t>Hawaiian Moons Natural Foods</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
@@ -2530,13 +2531,13 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G40" s="8" t="inlineStr"/>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>Tropical acai bowl + stock up on healthy snacks</t>
+          <t>Tropical acai bowl</t>
         </is>
       </c>
       <c r="I40" s="7" t="inlineStr">
@@ -2561,7 +2562,7 @@
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>Dinner at Monkeypod Kitchen (happy hour, live music)</t>
+          <t>Dinner at Monkeypod Kitchen</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -2571,7 +2572,7 @@
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
@@ -2606,7 +2607,7 @@
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>Molokini Crater snorkel boat tour (departs Ma'alaea)</t>
+          <t>Molokini Crater snorkel boat tour</t>
         </is>
       </c>
       <c r="E42" s="16" t="inlineStr">
@@ -2626,7 +2627,7 @@
       </c>
       <c r="H42" s="16" t="inlineStr">
         <is>
-          <t>⚠️ BOOK IN ADVANCE. Bring Dramamine (check w/ OB)</t>
+          <t>⚠️ BOOK IN ADVANCE. Bring Dramamine</t>
         </is>
       </c>
       <c r="I42" s="15" t="inlineStr">
@@ -2646,32 +2647,28 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>11:30 AM</t>
+          <t>10:30 AM</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Lunch at Coconut's Fish Cafe</t>
+          <t>Shave ice at Peace Love Shave Ice</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>Kihei</t>
+          <t>Azeka Plaza, Kihei</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
-        </is>
-      </c>
-      <c r="G43" s="9" t="inlineStr">
-        <is>
-          <t>Coconut's Fish Cafe</t>
-        </is>
-      </c>
+          <t>Food/Dining</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr"/>
       <c r="H43" s="8" t="inlineStr">
         <is>
-          <t>Cooked fish tacos — pregnancy safe</t>
+          <t>Post-snorkel treat!</t>
         </is>
       </c>
       <c r="I43" s="7" t="inlineStr">
@@ -2681,254 +2678,258 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="n">
+      <c r="A44" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B44" s="7" t="inlineStr">
+      <c r="B44" s="15" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>12:15 PM</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>Shave ice at Peace Love Shave Ice</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>Azeka Plaza, Kihei</t>
-        </is>
-      </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>Food / Dining</t>
-        </is>
-      </c>
-      <c r="G44" s="8" t="inlineStr"/>
-      <c r="H44" s="8" t="inlineStr">
-        <is>
-          <t>Organic syrups, Thai Iced Tea flavor, Roselani ice cream base</t>
-        </is>
-      </c>
-      <c r="I44" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
+      <c r="C44" s="15" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>Lunch at Mama's Fish House</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="inlineStr">
+        <is>
+          <t>Pa'ia</t>
+        </is>
+      </c>
+      <c r="F44" s="15" t="inlineStr">
+        <is>
+          <t>Must-Book</t>
+        </is>
+      </c>
+      <c r="G44" s="17" t="inlineStr">
+        <is>
+          <t>Mama's Fish House</t>
+        </is>
+      </c>
+      <c r="H44" s="16" t="inlineStr">
+        <is>
+          <t>✅ RESERVED 12:00 PM. Order cooked dishes for Brittany</t>
+        </is>
+      </c>
+      <c r="I44" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="18" t="n">
+      <c r="A45" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B45" s="18" t="inlineStr">
+      <c r="B45" s="10" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C45" s="18" t="inlineStr">
-        <is>
-          <t>1:00 PM</t>
-        </is>
-      </c>
-      <c r="D45" s="19" t="inlineStr">
-        <is>
-          <t>Visit Ahihi-Kinau Marine Preserve — tide pools &amp; lava fields</t>
-        </is>
-      </c>
-      <c r="E45" s="19" t="inlineStr">
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>2:00 – 4:30 PM</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>Beach relaxation or drive back for rest</t>
+        </is>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>Pa'ia / 2777 S Kihei Rd</t>
+        </is>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>Beach/Water</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr"/>
+      <c r="H45" s="11" t="inlineStr">
+        <is>
+          <t>Relax before luau. Nap if needed!</t>
+        </is>
+      </c>
+      <c r="I45" s="10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>Tue, May 5</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>5:45 PM</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>Old Lahaina Luau</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>1251 Front St, Lahaina</t>
+        </is>
+      </c>
+      <c r="F46" s="15" t="inlineStr">
+        <is>
+          <t>Must-Book</t>
+        </is>
+      </c>
+      <c r="G46" s="17" t="inlineStr">
+        <is>
+          <t>Old Lahaina Luau</t>
+        </is>
+      </c>
+      <c r="H46" s="16" t="inlineStr">
+        <is>
+          <t>✅ RESERVED 5:45 PM. Seated &amp; relaxed — perfect for pregnancy</t>
+        </is>
+      </c>
+      <c r="I46" s="15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>Wed, May 6</t>
+        </is>
+      </c>
+      <c r="C47" s="18" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>'Iao Valley State Monument</t>
+        </is>
+      </c>
+      <c r="E47" s="19" t="inlineStr">
+        <is>
+          <t>'Iao Valley</t>
+        </is>
+      </c>
+      <c r="F47" s="18" t="inlineStr">
+        <is>
+          <t>Nature/Hiking</t>
+        </is>
+      </c>
+      <c r="G47" s="20" t="inlineStr">
+        <is>
+          <t>'Iao Valley Info</t>
+        </is>
+      </c>
+      <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>Short paved path. Perfect for pregnancy</t>
+        </is>
+      </c>
+      <c r="I47" s="18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Wed, May 6</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>10:30 AM</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Lunch at Sam Sato's</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Wailuku</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>Food/Dining</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr"/>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>Famous local spot — the manju is a must!</t>
+        </is>
+      </c>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>Wed, May 6</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>12:00 PM</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>Ahihi-Kinau Marine Preserve</t>
+        </is>
+      </c>
+      <c r="E49" s="19" t="inlineStr">
         <is>
           <t>Wailea / La Perouse Bay</t>
         </is>
       </c>
-      <c r="F45" s="18" t="inlineStr">
-        <is>
-          <t>Nature / Hiking</t>
-        </is>
-      </c>
-      <c r="G45" s="19" t="inlineStr"/>
-      <c r="H45" s="19" t="inlineStr">
-        <is>
-          <t>Beautiful natural reserve. Gentle exploring, tide pools</t>
-        </is>
-      </c>
-      <c r="I45" s="18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="B46" s="10" t="inlineStr">
-        <is>
-          <t>Tue, May 5</t>
-        </is>
-      </c>
-      <c r="C46" s="10" t="inlineStr">
-        <is>
-          <t>2:30 – 4:30 PM</t>
-        </is>
-      </c>
-      <c r="D46" s="11" t="inlineStr">
-        <is>
-          <t>Beach relaxation at Big Beach (Makena State Park)</t>
-        </is>
-      </c>
-      <c r="E46" s="11" t="inlineStr">
-        <is>
-          <t>Makena</t>
-        </is>
-      </c>
-      <c r="F46" s="10" t="inlineStr">
-        <is>
-          <t>Beach / Water</t>
-        </is>
-      </c>
-      <c r="G46" s="11" t="inlineStr"/>
-      <c r="H46" s="11" t="inlineStr">
-        <is>
-          <t>Watch the bodyboarders! Brittany should wade gently — big shore break</t>
-        </is>
-      </c>
-      <c r="I46" s="10" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="B47" s="15" t="inlineStr">
-        <is>
-          <t>Tue, May 5</t>
-        </is>
-      </c>
-      <c r="C47" s="15" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="D47" s="16" t="inlineStr">
-        <is>
-          <t>Dinner at Mama's Fish House</t>
-        </is>
-      </c>
-      <c r="E47" s="16" t="inlineStr">
-        <is>
-          <t>Pa'ia</t>
-        </is>
-      </c>
-      <c r="F47" s="15" t="inlineStr">
-        <is>
-          <t>Must-Book</t>
-        </is>
-      </c>
-      <c r="G47" s="17" t="inlineStr">
-        <is>
-          <t>Mama's Fish House</t>
-        </is>
-      </c>
-      <c r="H47" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ RESERVE WELL IN ADVANCE. Order cooked dishes for Brittany</t>
-        </is>
-      </c>
-      <c r="I47" s="15" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="18" t="n">
-        <v>7</v>
-      </c>
-      <c r="B48" s="18" t="inlineStr">
-        <is>
-          <t>Wed, May 6</t>
-        </is>
-      </c>
-      <c r="C48" s="18" t="inlineStr">
-        <is>
-          <t>8:30 AM</t>
-        </is>
-      </c>
-      <c r="D48" s="19" t="inlineStr">
-        <is>
-          <t>'Iao Valley State Monument — 'Iao Needle viewpoint walk</t>
-        </is>
-      </c>
-      <c r="E48" s="19" t="inlineStr">
-        <is>
-          <t>'Iao Valley</t>
-        </is>
-      </c>
-      <c r="F48" s="18" t="inlineStr">
-        <is>
-          <t>Nature / Hiking</t>
-        </is>
-      </c>
-      <c r="G48" s="20" t="inlineStr">
-        <is>
-          <t>'Iao Valley Info</t>
-        </is>
-      </c>
-      <c r="H48" s="19" t="inlineStr">
-        <is>
-          <t>Short paved path. Perfect for pregnancy</t>
-        </is>
-      </c>
-      <c r="I48" s="18" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>Wed, May 6</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>10:30 AM</t>
-        </is>
-      </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>Lunch at Sam Sato's (dry mein and manju)</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>Wailuku</t>
-        </is>
-      </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>Food / Dining</t>
-        </is>
-      </c>
-      <c r="G49" s="8" t="inlineStr"/>
-      <c r="H49" s="8" t="inlineStr">
-        <is>
-          <t>Famous local spot — the manju is a must!</t>
-        </is>
-      </c>
-      <c r="I49" s="7" t="inlineStr">
+      <c r="F49" s="18" t="inlineStr">
+        <is>
+          <t>Nature/Hiking</t>
+        </is>
+      </c>
+      <c r="G49" s="19" t="inlineStr"/>
+      <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>Tide pools, lava fields. Gentle exploring</t>
+        </is>
+      </c>
+      <c r="I49" s="18" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2945,28 +2946,28 @@
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>12:00 – 4:00 PM</t>
+          <t>1:30 – 3:30 PM</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Beach relaxation or Wailea Beach Path walk</t>
+          <t>Beach relaxation at Big Beach or Kamaole</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>Wailea / Kihei</t>
+          <t>Makena / Kihei</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G50" s="11" t="inlineStr"/>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>Flat oceanfront path or lazy afternoon at the beach</t>
+          <t>Wade gently at Big Beach — big shore break</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr">
@@ -2991,12 +2992,12 @@
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>Luau — Old Lahaina Luau or Feast at Lele</t>
+          <t>Ka'anapali Sunset Sail Tour</t>
         </is>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>Lahaina</t>
+          <t>Ka'anapali Beach, Sheraton</t>
         </is>
       </c>
       <c r="F51" s="15" t="inlineStr">
@@ -3004,19 +3005,15 @@
           <t>Must-Book</t>
         </is>
       </c>
-      <c r="G51" s="17" t="inlineStr">
-        <is>
-          <t>Old Lahaina Luau</t>
-        </is>
-      </c>
+      <c r="G51" s="16" t="inlineStr"/>
       <c r="H51" s="16" t="inlineStr">
         <is>
-          <t>⚠️ BOOK IN ADVANCE. Seated &amp; relaxed — perfect for pregnancy</t>
+          <t>✅ RESERVED 5:00 PM. Departs from Sheraton beach</t>
         </is>
       </c>
       <c r="I51" s="15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3033,7 @@
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Easy morning walk along Wailea Beach Path</t>
+          <t>Walk along Wailea Beach Path</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
@@ -3046,13 +3043,13 @@
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G52" s="11" t="inlineStr"/>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>Flat oceanfront path, gorgeous views. Great gentle exercise</t>
+          <t>Flat oceanfront path, gorgeous views</t>
         </is>
       </c>
       <c r="I52" s="10" t="inlineStr">
@@ -3077,7 +3074,7 @@
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>Acai bowl at Brekkie Bowls food truck</t>
+          <t>Acai bowl at Brekkie Bowls</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -3087,13 +3084,13 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G53" s="8" t="inlineStr"/>
       <c r="H53" s="8" t="inlineStr">
         <is>
-          <t>Superfood acai bowl — perfect pregnancy fuel!</t>
+          <t>Superfood acai bowl</t>
         </is>
       </c>
       <c r="I53" s="7" t="inlineStr">
@@ -3118,17 +3115,17 @@
       </c>
       <c r="D54" s="8" t="inlineStr">
         <is>
-          <t>Shave ice at Ululani's (Kihei location)</t>
+          <t>Shave ice at Ululani's (Kihei)</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>61 S Kihei Rd, Kihei</t>
+          <t>61 S Kihei Rd</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G54" s="9" t="inlineStr">
@@ -3138,7 +3135,7 @@
       </c>
       <c r="H54" s="8" t="inlineStr">
         <is>
-          <t>Round 2! Try a different flavor combo</t>
+          <t>Round 2!</t>
         </is>
       </c>
       <c r="I54" s="7" t="inlineStr">
@@ -3163,7 +3160,7 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>Fresh fruit bowls at Maui Fruit Ninja</t>
+          <t>Fresh fruit at Maui Fruit Ninja</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -3173,7 +3170,7 @@
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G55" s="9" t="inlineStr">
@@ -3183,7 +3180,7 @@
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>Seasonal tropical fruit bowls &amp; dairy-free sorbets</t>
+          <t>Tropical fruit bowls</t>
         </is>
       </c>
       <c r="I55" s="7" t="inlineStr">
@@ -3208,7 +3205,7 @@
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Beach time + revisits, shopping, souvenirs</t>
+          <t>Beach time + shopping, souvenirs</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
@@ -3218,13 +3215,13 @@
       </c>
       <c r="F56" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G56" s="11" t="inlineStr"/>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>Last full beach day! Soak it in</t>
+          <t>Last full beach day!</t>
         </is>
       </c>
       <c r="I56" s="10" t="inlineStr">
@@ -3249,23 +3246,23 @@
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>Pie &amp; treats at Leoda's Kitchen and Pie Shop</t>
+          <t>Leoda's Kitchen and Pie Shop</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>820 Olowalu Village Rd, Lahaina</t>
+          <t>820 Olowalu Village Rd</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Food / Dining</t>
+          <t>Food/Dining</t>
         </is>
       </c>
       <c r="G57" s="8" t="inlineStr"/>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>Famous pies — banana cream, macnut, savory pot pies</t>
+          <t>Famous pies</t>
         </is>
       </c>
       <c r="I57" s="7" t="inlineStr">
@@ -3310,7 +3307,7 @@
       </c>
       <c r="H58" s="16" t="inlineStr">
         <is>
-          <t>BOOKED — hoping for outdoor 5:30 seating (waitlisted). Keep checking!</t>
+          <t>BOOKED — hoping for outdoor 5:30 (waitlisted)</t>
         </is>
       </c>
       <c r="I58" s="15" t="inlineStr">
@@ -3335,7 +3332,7 @@
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>Last morning beach walk at Kamaole Beach</t>
+          <t>Last morning beach walk</t>
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr">
@@ -3345,7 +3342,7 @@
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t>Beach / Water</t>
+          <t>Beach/Water</t>
         </is>
       </c>
       <c r="G59" s="11" t="inlineStr"/>
@@ -3376,7 +3373,7 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Pack up &amp; check out of Airbnb by 11 AM. Return rental car.</t>
+          <t>Pack up &amp; check out by 11 AM. Return rental car.</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -3392,7 +3389,7 @@
       <c r="G60" s="5" t="inlineStr"/>
       <c r="H60" s="5" t="inlineStr">
         <is>
-          <t>Airbnb check-out: 11:00 AM. Airport is ~25 min from Kihei</t>
+          <t>Airbnb check-out: 11:00 AM. Airport ~25 min</t>
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr">
@@ -3439,7 +3436,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I2:I60">
+  <conditionalFormatting sqref="I2:I61">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Y"</formula>
     </cfRule>
@@ -3460,15 +3457,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G46" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G47" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G50" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G53" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G57" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G54" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G55" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G58" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3481,7 +3477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B67"/>
+  <dimension ref="A1:B68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3603,7 +3599,7 @@
     <row r="12">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>• Avoid raw fish/sushi (ahi poke) — order cooked fish dishes</t>
+          <t>• Avoid raw fish/sushi (ahi poke) — order cooked fish</t>
         </is>
       </c>
       <c r="B12" s="22" t="n"/>
@@ -3611,7 +3607,7 @@
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>• Avoid scuba diving, zip-lining, parasailing, horseback riding</t>
+          <t>• Avoid scuba, zip-lining, parasailing, horseback riding</t>
         </is>
       </c>
       <c r="B13" s="22" t="n"/>
@@ -3619,7 +3615,7 @@
     <row r="14">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>• Snorkeling is generally OK — check with OB first</t>
+          <t>• Snorkeling generally OK — check with OB first</t>
         </is>
       </c>
       <c r="B14" s="22" t="n"/>
@@ -3627,7 +3623,7 @@
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t>• Haleakala summit: thin air, limit time to ~30 min, leave if dizzy</t>
+          <t>• Haleakala summit: thin air, limit to ~30 min, leave if dizzy</t>
         </is>
       </c>
       <c r="B15" s="22" t="n"/>
@@ -3635,7 +3631,7 @@
     <row r="16">
       <c r="A16" s="25" t="inlineStr">
         <is>
-          <t>• Stay hydrated — bring water everywhere, seek shade often</t>
+          <t>• Stay hydrated — extra water, seek shade often</t>
         </is>
       </c>
       <c r="B16" s="22" t="n"/>
@@ -3643,7 +3639,7 @@
     <row r="17">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>• Dramamine for boat/car sickness — check with OB for pregnancy-safe brand</t>
+          <t>• Dramamine for boat/car — check with OB for pregnancy-safe brand</t>
         </is>
       </c>
       <c r="B17" s="22" t="n"/>
@@ -3651,7 +3647,7 @@
     <row r="18">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>• Road to Hana: take breaks often, go slow, carry snacks (helps nausea)</t>
+          <t>• Road to Hana: take breaks, go slow, carry snacks (nausea)</t>
         </is>
       </c>
       <c r="B18" s="22" t="n"/>
@@ -3659,7 +3655,7 @@
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>• Big Beach (Makena): watch shore break — wade gently, don't bodyboard</t>
+          <t>• Big Beach: watch shore break — wade gently</t>
         </is>
       </c>
       <c r="B19" s="22" t="n"/>
@@ -3667,7 +3663,7 @@
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>• Prenatal massage: request pregnancy-trained masseuse (2nd/3rd trimester only)</t>
+          <t>• Prenatal massage: request pregnancy-trained masseuse</t>
         </is>
       </c>
       <c r="B20" s="22" t="n"/>
@@ -3675,7 +3671,7 @@
     <row r="21">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>• Book an aisle seat on the plane for bathroom access</t>
+          <t>• Aisle seat on plane for bathroom access</t>
         </is>
       </c>
       <c r="B21" s="22" t="n"/>
@@ -3683,7 +3679,7 @@
     <row r="22">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>• Wear compression socks for flights to prevent swelling</t>
+          <t>• Compression socks for flights to prevent swelling</t>
         </is>
       </c>
       <c r="B22" s="22" t="n"/>
@@ -3691,7 +3687,7 @@
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
-          <t>⚠️ MUST-BOOK IN ADVANCE ITEMS</t>
+          <t>⚠️ MUST-BOOK / RESERVED ITEMS</t>
         </is>
       </c>
       <c r="B24" s="22" t="n"/>
@@ -3704,19 +3700,19 @@
       </c>
       <c r="B25" s="27" t="inlineStr">
         <is>
-          <t>https://www.recreation.gov/ticket/facility/253731</t>
+          <t>⚠️ Book — https://www.recreation.gov/ticket/facility/253731</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>Wai'anapanapa State Park Entry</t>
+          <t>Wai'anapanapa State Park</t>
         </is>
       </c>
       <c r="B26" s="27" t="inlineStr">
         <is>
-          <t>https://www.gowaianapanapa.com/</t>
+          <t>✅ RESERVED 12:30–3 PM — https://www.gowaianapanapa.com/</t>
         </is>
       </c>
     </row>
@@ -3728,198 +3724,202 @@
       </c>
       <c r="B27" s="27" t="inlineStr">
         <is>
-          <t>https://www.pacificwhale.org/cruises/molokini-snorkel/</t>
+          <t>⚠️ Book — https://www.pacificwhale.org/cruises/molokini-snorkel/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="26" t="inlineStr">
         <is>
-          <t>Mama's Fish House Dinner</t>
+          <t>Mama's Fish House — Tue May 5</t>
         </is>
       </c>
       <c r="B28" s="27" t="inlineStr">
         <is>
-          <t>https://www.mamasfishhouse.com/</t>
+          <t>✅ RESERVED 12:00 PM — https://www.mamasfishhouse.com/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="26" t="inlineStr">
         <is>
-          <t>Old Lahaina Luau</t>
+          <t>Old Lahaina Luau — Tue May 5</t>
         </is>
       </c>
       <c r="B29" s="27" t="inlineStr">
         <is>
-          <t>https://www.oldlahainaluau.com/</t>
+          <t>✅ RESERVED 5:45 PM — https://www.oldlahainaluau.com/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="26" t="inlineStr">
         <is>
-          <t>Merriman's Kapalua (BOOKED — waitlist outdoor 5:30)</t>
-        </is>
-      </c>
-      <c r="B30" s="27" t="inlineStr">
-        <is>
-          <t>https://www.merrimanshawaii.com/kapalua/</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="21" t="inlineStr">
+          <t>Ka'anapali Sunset Sail — Wed May 6</t>
+        </is>
+      </c>
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>✅ RESERVED 5:00 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>Merriman's Kapalua — Thu May 7</t>
+        </is>
+      </c>
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>BOOKED (waitlist outdoor 5:30) — https://www.merrimanshawaii.com/kapalua/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
         <is>
           <t>🍧 SHAVED ICE / ACAI / FRUIT SPOTS</t>
         </is>
       </c>
-      <c r="B32" s="22" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="28" t="inlineStr">
+      <c r="B33" s="22" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="29" t="inlineStr">
         <is>
           <t>Ululani's Hawaiian Shave Ice</t>
         </is>
       </c>
-      <c r="B33" s="25" t="inlineStr">
-        <is>
-          <t>Kihei (61 S Kihei Rd), Kahului, Wailuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="28" t="inlineStr">
+      <c r="B34" s="25" t="inlineStr">
+        <is>
+          <t>Kihei, Kahului, Wailuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
         <is>
           <t>Peace Love Shave Ice</t>
         </is>
       </c>
-      <c r="B34" s="25" t="inlineStr">
-        <is>
-          <t>Azeka Plaza, Kihei — organic syrups, Thai Iced Tea flavor</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="28" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
+        <is>
+          <t>Azeka Plaza, Kihei</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="inlineStr">
         <is>
           <t>Surfing Monkey Shave Ice</t>
         </is>
       </c>
-      <c r="B35" s="25" t="inlineStr">
-        <is>
-          <t>Kihei — Kona coffee flavor, vegan coconut milk ice cream</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="28" t="inlineStr">
+      <c r="B36" s="25" t="inlineStr">
+        <is>
+          <t>Kihei — Kona coffee flavor</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="inlineStr">
         <is>
           <t>Halfway to Hana</t>
         </is>
       </c>
-      <c r="B36" s="25" t="inlineStr">
-        <is>
-          <t>Haiku — shave ice + banana bread on Hana Hwy</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="28" t="inlineStr">
-        <is>
-          <t>Mo'Ono Hawaii (food truck)</t>
-        </is>
-      </c>
       <c r="B37" s="25" t="inlineStr">
         <is>
-          <t>Kahului — acai bowls, fresh fruit toppings</t>
+          <t>Haiku — shave ice + banana bread</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="28" t="inlineStr">
-        <is>
-          <t>Brekkie Bowls (food truck)</t>
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>Mo'Ono Hawaii</t>
         </is>
       </c>
       <c r="B38" s="25" t="inlineStr">
         <is>
+          <t>Kahului — acai bowls</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>Brekkie Bowls</t>
+        </is>
+      </c>
+      <c r="B39" s="25" t="inlineStr">
+        <is>
           <t>Wailea — superfood acai bowls</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="28" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="29" t="inlineStr">
         <is>
           <t>Hawaiian Moons Natural Foods</t>
         </is>
       </c>
-      <c r="B39" s="25" t="inlineStr">
-        <is>
-          <t>Kihei — tropical acai bowl + healthy groceries</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="28" t="inlineStr">
+      <c r="B40" s="25" t="inlineStr">
+        <is>
+          <t>Kihei — acai + healthy groceries</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="29" t="inlineStr">
         <is>
           <t>Wow Wow Hawaiian Lemonade</t>
         </is>
       </c>
-      <c r="B40" s="25" t="inlineStr">
-        <is>
-          <t>Kihei — acai bowls + fresh lemonades</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="28" t="inlineStr">
+      <c r="B41" s="25" t="inlineStr">
+        <is>
+          <t>Kihei — acai + fresh lemonades</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="29" t="inlineStr">
         <is>
           <t>Maui Fruit Ninja</t>
         </is>
       </c>
-      <c r="B41" s="25" t="inlineStr">
-        <is>
-          <t>Lahaina — seasonal fresh fruit bowls &amp; dairy-free sorbets</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="28" t="inlineStr">
+      <c r="B42" s="25" t="inlineStr">
+        <is>
+          <t>Lahaina — tropical fruit bowls</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="29" t="inlineStr">
         <is>
           <t>Leoda's Kitchen &amp; Pie Shop</t>
         </is>
       </c>
-      <c r="B42" s="25" t="inlineStr">
-        <is>
-          <t>820 Olowalu Village Rd — pies, pastries, savory pot pies</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="28" t="inlineStr">
+      <c r="B43" s="25" t="inlineStr">
+        <is>
+          <t>820 Olowalu Village Rd — pies</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="29" t="inlineStr">
         <is>
           <t>Ahihi-Kinau Marine Preserve</t>
         </is>
       </c>
-      <c r="B43" s="25" t="inlineStr">
-        <is>
-          <t>South Maui / La Perouse Bay — tide pools, lava fields</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="21" t="inlineStr">
+      <c r="B44" s="25" t="inlineStr">
+        <is>
+          <t>South Maui — tide pools, lava fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="21" t="inlineStr">
         <is>
           <t>🧳 PACKING REMINDERS</t>
-        </is>
-      </c>
-      <c r="B45" s="22" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="25" t="inlineStr">
-        <is>
-          <t>☐ Reef-safe sunscreen (required by Hawaii law)</t>
         </is>
       </c>
       <c r="B46" s="22" t="n"/>
@@ -3927,7 +3927,7 @@
     <row r="47">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>☐ Snorkel gear (or rent on island)</t>
+          <t>☐ Reef-safe sunscreen (required by Hawaii law)</t>
         </is>
       </c>
       <c r="B47" s="22" t="n"/>
@@ -3935,7 +3935,7 @@
     <row r="48">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>☐ Comfortable walking shoes</t>
+          <t>☐ Snorkel gear (or rent)</t>
         </is>
       </c>
       <c r="B48" s="22" t="n"/>
@@ -3943,7 +3943,7 @@
     <row r="49">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>☐ Warm layers for Haleakala sunrise (30-40°F at summit)</t>
+          <t>☐ Comfortable walking shoes</t>
         </is>
       </c>
       <c r="B49" s="22" t="n"/>
@@ -3951,7 +3951,7 @@
     <row r="50">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>☐ Rain jacket (Road to Hana gets wet)</t>
+          <t>☐ Warm layers for Haleakala (30-40°F)</t>
         </is>
       </c>
       <c r="B50" s="22" t="n"/>
@@ -3959,7 +3959,7 @@
     <row r="51">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>☐ Water shoes (rocky beaches)</t>
+          <t>☐ Rain jacket (Hana gets wet)</t>
         </is>
       </c>
       <c r="B51" s="22" t="n"/>
@@ -3967,7 +3967,7 @@
     <row r="52">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>☐ Swimsuits &amp; rash guards</t>
+          <t>☐ Water shoes</t>
         </is>
       </c>
       <c r="B52" s="22" t="n"/>
@@ -3975,7 +3975,7 @@
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>☐ Reusable water bottles (HYDRATE — extra for pregnancy!)</t>
+          <t>☐ Swimsuits &amp; rash guards</t>
         </is>
       </c>
       <c r="B53" s="22" t="n"/>
@@ -3983,7 +3983,7 @@
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>☐ Portable charger / power bank</t>
+          <t>☐ Reusable water bottles (HYDRATE!)</t>
         </is>
       </c>
       <c r="B54" s="22" t="n"/>
@@ -3991,7 +3991,7 @@
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>☐ Car phone mount for Hana drive</t>
+          <t>☐ Portable charger</t>
         </is>
       </c>
       <c r="B55" s="22" t="n"/>
@@ -3999,7 +3999,7 @@
     <row r="56">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>☐ Dramamine (check w/ OB for pregnancy-safe option)</t>
+          <t>☐ Car phone mount for Hana</t>
         </is>
       </c>
       <c r="B56" s="22" t="n"/>
@@ -4007,7 +4007,7 @@
     <row r="57">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>☐ Dry bag for water activities</t>
+          <t>☐ Dramamine (check w/ OB)</t>
         </is>
       </c>
       <c r="B57" s="22" t="n"/>
@@ -4015,7 +4015,7 @@
     <row r="58">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>☐ Compression socks for flights</t>
+          <t>☐ Dry bag</t>
         </is>
       </c>
       <c r="B58" s="22" t="n"/>
@@ -4023,7 +4023,7 @@
     <row r="59">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>☐ Prenatal vitamins &amp; pregnancy meds</t>
+          <t>☐ Compression socks</t>
         </is>
       </c>
       <c r="B59" s="22" t="n"/>
@@ -4031,7 +4031,7 @@
     <row r="60">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>☐ Pregnancy pillow or support wedge</t>
+          <t>☐ Prenatal vitamins &amp; meds</t>
         </is>
       </c>
       <c r="B60" s="22" t="n"/>
@@ -4039,62 +4039,70 @@
     <row r="61">
       <c r="A61" s="25" t="inlineStr">
         <is>
+          <t>☐ Pregnancy pillow</t>
+        </is>
+      </c>
+      <c r="B61" s="22" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
           <t>☐ Snacks for Hana (crackers, fruit, nuts)</t>
         </is>
       </c>
-      <c r="B61" s="22" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="21" t="inlineStr">
+      <c r="B62" s="22" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="21" t="inlineStr">
         <is>
           <t>🚨 EMERGENCY CONTACTS</t>
         </is>
       </c>
-      <c r="B63" s="22" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="23" t="inlineStr">
-        <is>
-          <t>Maui Memorial Medical Center</t>
-        </is>
-      </c>
-      <c r="B64" s="24" t="inlineStr">
-        <is>
-          <t>(808) 244-9056</t>
-        </is>
-      </c>
+      <c r="B64" s="22" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="23" t="inlineStr">
         <is>
-          <t>Maui Police (non-emergency)</t>
+          <t>Maui Memorial Medical Center</t>
         </is>
       </c>
       <c r="B65" s="24" t="inlineStr">
         <is>
-          <t>(808) 244-6400</t>
+          <t>(808) 244-9056</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="23" t="inlineStr">
         <is>
-          <t>Hawaii Visitor Emergency Line</t>
+          <t>Maui Police (non-emergency)</t>
         </is>
       </c>
       <c r="B66" s="24" t="inlineStr">
         <is>
-          <t>911</t>
+          <t>(808) 244-6400</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="23" t="inlineStr">
         <is>
+          <t>Hawaii Visitor Emergency Line</t>
+        </is>
+      </c>
+      <c r="B67" s="24" t="inlineStr">
+        <is>
+          <t>911</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="23" t="inlineStr">
+        <is>
           <t>Poison Control</t>
         </is>
       </c>
-      <c r="B67" s="24" t="inlineStr">
+      <c r="B68" s="24" t="inlineStr">
         <is>
           <t>1-800-222-1222</t>
         </is>
@@ -4106,11 +4114,11 @@
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A64:B64"/>
     <mergeCell ref="A60:B60"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A49:B49"/>
     <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A45:B45"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A61:B61"/>
     <mergeCell ref="A16:B16"/>
@@ -4123,16 +4131,16 @@
     <mergeCell ref="A50:B50"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A33:B33"/>
     <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A32:B32"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A53:B53"/>
+    <mergeCell ref="A62:B62"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A52:B52"/>
     <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A63:B63"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A58:B58"/>
   </mergeCells>
@@ -4142,7 +4150,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Replace Molokini boat tour with beach snorkel at Ulua Beach, update Haleakala to last-minute tickets
- Day 6: Self-guided snorkel at Ulua Beach (free, no boat, pregnancy-friendly)
- Day 3: Haleakala note updated — book 2-day-ahead last-minute tickets on recreation.gov

Co-Authored-By: Claude (claude-opus-4-6[1m]) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/maui_itinerary.xlsx
+++ b/maui_itinerary.xlsx
@@ -1500,7 +1500,7 @@
       </c>
       <c r="H15" s="16" t="inlineStr">
         <is>
-          <t>⚠️ MUST RESERVE. Sunrise ~5:50 AM. Warm layers!</t>
+          <t>⚠️ LAST-MINUTE TICKETS: Book 2 days ahead on recreation.gov (drops midnight ET). Try Apr 30 for May 2. Warm layers!</t>
         </is>
       </c>
       <c r="I15" s="15" t="inlineStr">
@@ -2592,45 +2592,41 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="15" t="n">
+      <c r="A42" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B42" s="15" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>Tue, May 5</t>
         </is>
       </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>6:00 AM</t>
-        </is>
-      </c>
-      <c r="D42" s="16" t="inlineStr">
-        <is>
-          <t>Molokini Crater snorkel boat tour</t>
-        </is>
-      </c>
-      <c r="E42" s="16" t="inlineStr">
-        <is>
-          <t>Ma'alaea Harbor</t>
-        </is>
-      </c>
-      <c r="F42" s="15" t="inlineStr">
-        <is>
-          <t>Must-Book</t>
-        </is>
-      </c>
-      <c r="G42" s="17" t="inlineStr">
-        <is>
-          <t>Pacific Whale Foundation</t>
-        </is>
-      </c>
-      <c r="H42" s="16" t="inlineStr">
-        <is>
-          <t>⚠️ BOOK IN ADVANCE. Bring Dramamine</t>
-        </is>
-      </c>
-      <c r="I42" s="15" t="inlineStr">
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>8:30 – 10:30 AM</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>Self-guided snorkel at Ulua Beach (turtles, reef fish)</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>Ulua Beach, Wailea</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>Beach / Water</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr"/>
+      <c r="H42" s="11" t="inlineStr">
+        <is>
+          <t>Free! Calm water, turtles. Bring gear or rent. No boat = no seasickness</t>
+        </is>
+      </c>
+      <c r="I42" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2647,7 +2643,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>10:30 AM</t>
+          <t>10:45 AM</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
@@ -3588,6 +3584,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
@@ -3684,6 +3681,7 @@
       </c>
       <c r="B22" s="22" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
@@ -3719,12 +3717,12 @@
     <row r="27">
       <c r="A27" s="26" t="inlineStr">
         <is>
-          <t>Molokini Snorkel Tour</t>
+          <t>Haleakala Sunrise (last-minute tickets)</t>
         </is>
       </c>
       <c r="B27" s="27" t="inlineStr">
         <is>
-          <t>⚠️ Book — https://www.pacificwhale.org/cruises/molokini-snorkel/</t>
+          <t>⚠️ Try 2 days ahead on recreation.gov — https://www.recreation.gov/ticket/facility/253731</t>
         </is>
       </c>
     </row>
@@ -4112,9 +4110,9 @@
   <mergeCells count="33">
     <mergeCell ref="A48:B48"/>
     <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A59:B59"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A64:B64"/>
     <mergeCell ref="A60:B60"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A49:B49"/>

</xml_diff>